<commit_message>
fix(azure): add api_version field to credential form (WBS 3.5)
Azure OpenAI requires an API version; the UI had no field so credentials
saved without it and inference failed. Add Azure-only input, wire create/
update payloads (null-clear on edit), i18n across locales, and mark WBS 3.5 Done.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/commercialization/Open-Notebook-Commercialization-WBS-Task-Schedule.xlsx
+++ b/docs/commercialization/Open-Notebook-Commercialization-WBS-Task-Schedule.xlsx
@@ -760,13 +760,13 @@
         <v>32</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>4</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.0625</v>
+        <v>0.3125</v>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
@@ -1032,10 +1032,10 @@
         <v>880</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>0.2006818181818182</v>
+        <v>0.2097727272727273</v>
       </c>
     </row>
     <row r="20">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="B22" s="11" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="23">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="B24" s="11" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25">
@@ -1102,7 +1102,7 @@
         </is>
       </c>
       <c r="B26" s="11" t="n">
-        <v>703.4</v>
+        <v>695.4</v>
       </c>
     </row>
     <row r="27">
@@ -1112,7 +1112,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>88.2</v>
+        <v>87.2</v>
       </c>
     </row>
     <row r="28">
@@ -3831,9 +3831,9 @@
           <t>Working Azure credential UI</t>
         </is>
       </c>
-      <c r="F36" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F36" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G36" s="16" t="inlineStr">
@@ -3852,9 +3852,11 @@
       <c r="J36" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="K36" s="17" t="n"/>
+      <c r="K36" s="17" t="n">
+        <v>4</v>
+      </c>
       <c r="L36" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M36" s="3" t="inlineStr">
         <is>
@@ -3867,7 +3869,9 @@
       <c r="O36" s="19" t="n">
         <v>46239</v>
       </c>
-      <c r="P36" s="3" t="n"/>
+      <c r="P36" s="19" t="n">
+        <v>46234</v>
+      </c>
       <c r="Q36" s="3" t="inlineStr">
         <is>
           <t>User can set api_version in UI; connection + inference succeed</t>
@@ -3875,12 +3879,12 @@
       </c>
       <c r="R36" s="3" t="inlineStr">
         <is>
-          <t>PR #6 nested STT config kept; esperanto#263 transcription format fixed via task 3.4</t>
+          <t>Azure-only field; required on create; null-clear on edit via buildCredentialUpdatePayload</t>
         </is>
       </c>
       <c r="S36" s="3" t="inlineStr">
         <is>
-          <t>Bug found 2026-07-22</t>
+          <t>CredentialFormDialog + credential-update-payload + i18n (14 locales)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(wp2): close Entra auth with ownership, admin UI, and catalog ACL
Land remaining WP2 work: RecordID/session hardening, transformation shared vs personal ownership with soft-delete builtins, meaningful 403 messages, admin-only nav/routes, and WBS 4.0–4.14 marked Done.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/commercialization/Open-Notebook-Commercialization-WBS-Task-Schedule.xlsx
+++ b/docs/commercialization/Open-Notebook-Commercialization-WBS-Task-Schedule.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimating Assumptions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'WBS Task List'!$A$5:$S$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'WBS Task List'!$A$5:$S$93</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -138,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -196,9 +196,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -817,18 +814,16 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>156</v>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>181</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>181</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>19.5</v>
+        <v>22.6</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.003846153846153846</v>
+        <v>1</v>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
@@ -1029,13 +1024,13 @@
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>880</v>
+        <v>905</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>186</v>
+        <v>367</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>0.2097727272727273</v>
+        <v>0.4033149171270718</v>
       </c>
     </row>
     <row r="20">
@@ -1052,7 +1047,7 @@
         </is>
       </c>
       <c r="B21" s="11" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22">
@@ -1062,7 +1057,7 @@
         </is>
       </c>
       <c r="B22" s="11" t="n">
-        <v>31</v>
+        <v>46</v>
       </c>
     </row>
     <row r="23">
@@ -1072,7 +1067,7 @@
         </is>
       </c>
       <c r="B23" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1082,7 +1077,7 @@
         </is>
       </c>
       <c r="B24" s="11" t="n">
-        <v>51</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25">
@@ -1102,7 +1097,7 @@
         </is>
       </c>
       <c r="B26" s="11" t="n">
-        <v>695.4</v>
+        <v>540</v>
       </c>
     </row>
     <row r="27">
@@ -1112,7 +1107,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>87.2</v>
+        <v>67.8</v>
       </c>
     </row>
     <row r="28">
@@ -1182,7 +1177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S89"/>
+  <dimension ref="A1:S93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4394,9 +4389,9 @@
           <t>Branch + spike notes / Entra checklist</t>
         </is>
       </c>
-      <c r="F43" s="25" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="F43" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G43" s="20" t="inlineStr">
@@ -4415,9 +4410,11 @@
       <c r="J43" s="17" t="n">
         <v>0.5</v>
       </c>
-      <c r="K43" s="17" t="n"/>
+      <c r="K43" s="17" t="n">
+        <v>4</v>
+      </c>
       <c r="L43" s="18" t="n">
-        <v>0.15</v>
+        <v>1</v>
       </c>
       <c r="M43" s="3" t="inlineStr">
         <is>
@@ -4430,7 +4427,9 @@
       <c r="O43" s="19" t="n">
         <v>46235</v>
       </c>
-      <c r="P43" s="3" t="n"/>
+      <c r="P43" s="19" t="n">
+        <v>46239</v>
+      </c>
       <c r="Q43" s="3" t="inlineStr">
         <is>
           <t>Branch ready; Entra app registration checklist drafted</t>
@@ -4438,12 +4437,12 @@
       </c>
       <c r="R43" s="3" t="inlineStr">
         <is>
-          <t>Current work package kickoff</t>
+          <t>Kickoff complete; WP2 implemented on wp-2-entra-auth</t>
         </is>
       </c>
       <c r="S43" s="3" t="inlineStr">
         <is>
-          <t>Plan WP2; CLAUDE.md current WP = WP2</t>
+          <t>branch wp-2-entra-auth</t>
         </is>
       </c>
     </row>
@@ -4474,9 +4473,9 @@
           <t>api/auth/ + PasswordAuthProvider</t>
         </is>
       </c>
-      <c r="F44" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F44" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G44" s="20" t="inlineStr">
@@ -4495,9 +4494,11 @@
       <c r="J44" s="17" t="n">
         <v>1.5</v>
       </c>
-      <c r="K44" s="17" t="n"/>
+      <c r="K44" s="17" t="n">
+        <v>12</v>
+      </c>
       <c r="L44" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M44" s="3" t="inlineStr">
         <is>
@@ -4510,7 +4511,9 @@
       <c r="O44" s="19" t="n">
         <v>46238</v>
       </c>
-      <c r="P44" s="3" t="n"/>
+      <c r="P44" s="19" t="n">
+        <v>46239</v>
+      </c>
       <c r="Q44" s="3" t="inlineStr">
         <is>
           <t>Password provider still works as local-dev fallback behind a flag</t>
@@ -4521,7 +4524,11 @@
           <t>Preserve existing password behaviour for tests</t>
         </is>
       </c>
-      <c r="S44" s="3" t="inlineStr"/>
+      <c r="S44" s="3" t="inlineStr">
+        <is>
+          <t>api/auth/; PasswordAuthProvider</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="75" customHeight="1">
       <c r="A45" s="3" t="inlineStr">
@@ -4550,9 +4557,9 @@
           <t>EntraOIDCProvider</t>
         </is>
       </c>
-      <c r="F45" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F45" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G45" s="20" t="inlineStr">
@@ -4571,9 +4578,11 @@
       <c r="J45" s="17" t="n">
         <v>2.5</v>
       </c>
-      <c r="K45" s="17" t="n"/>
+      <c r="K45" s="17" t="n">
+        <v>20</v>
+      </c>
       <c r="L45" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M45" s="3" t="inlineStr">
         <is>
@@ -4586,7 +4595,9 @@
       <c r="O45" s="19" t="n">
         <v>46241</v>
       </c>
-      <c r="P45" s="3" t="n"/>
+      <c r="P45" s="19" t="n">
+        <v>46239</v>
+      </c>
       <c r="Q45" s="3" t="inlineStr">
         <is>
           <t>API accepts valid Entra JWTs and rejects invalid/expired ones</t>
@@ -4597,7 +4608,11 @@
           <t>Use maintained JWT/JWKS libraries</t>
         </is>
       </c>
-      <c r="S45" s="3" t="inlineStr"/>
+      <c r="S45" s="3" t="inlineStr">
+        <is>
+          <t>api/auth/entra.py</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="75" customHeight="1">
       <c r="A46" s="3" t="inlineStr">
@@ -4626,9 +4641,9 @@
           <t>AuthMiddleware</t>
         </is>
       </c>
-      <c r="F46" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F46" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G46" s="20" t="inlineStr">
@@ -4647,9 +4662,11 @@
       <c r="J46" s="17" t="n">
         <v>1.5</v>
       </c>
-      <c r="K46" s="17" t="n"/>
+      <c r="K46" s="17" t="n">
+        <v>12</v>
+      </c>
       <c r="L46" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M46" s="3" t="inlineStr">
         <is>
@@ -4662,14 +4679,20 @@
       <c r="O46" s="19" t="n">
         <v>46242</v>
       </c>
-      <c r="P46" s="3" t="n"/>
+      <c r="P46" s="19" t="n">
+        <v>46239</v>
+      </c>
       <c r="Q46" s="3" t="inlineStr">
         <is>
           <t>Every protected API request validates a real Entra token when entra mode is on</t>
         </is>
       </c>
       <c r="R46" s="3" t="inlineStr"/>
-      <c r="S46" s="3" t="inlineStr"/>
+      <c r="S46" s="3" t="inlineStr">
+        <is>
+          <t>api/auth/middleware.py; session + CSRF</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="75" customHeight="1">
       <c r="A47" s="3" t="inlineStr">
@@ -4698,9 +4721,9 @@
           <t>user model + migration</t>
         </is>
       </c>
-      <c r="F47" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F47" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G47" s="20" t="inlineStr">
@@ -4719,9 +4742,11 @@
       <c r="J47" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="K47" s="17" t="n"/>
+      <c r="K47" s="17" t="n">
+        <v>16</v>
+      </c>
       <c r="L47" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M47" s="3" t="inlineStr">
         <is>
@@ -4734,7 +4759,9 @@
       <c r="O47" s="19" t="n">
         <v>46245</v>
       </c>
-      <c r="P47" s="3" t="n"/>
+      <c r="P47" s="19" t="n">
+        <v>46239</v>
+      </c>
       <c r="Q47" s="3" t="inlineStr">
         <is>
           <t>User record exists after first successful login</t>
@@ -4745,7 +4772,11 @@
           <t>Migrations are hard-coded, not auto-discovered</t>
         </is>
       </c>
-      <c r="S47" s="3" t="inlineStr"/>
+      <c r="S47" s="3" t="inlineStr">
+        <is>
+          <t>migration 24 user/session schema</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="75" customHeight="1">
       <c r="A48" s="3" t="inlineStr">
@@ -4774,9 +4805,9 @@
           <t>RBAC checks on sensitive routers</t>
         </is>
       </c>
-      <c r="F48" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F48" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G48" s="16" t="inlineStr">
@@ -4795,9 +4826,11 @@
       <c r="J48" s="17" t="n">
         <v>1.5</v>
       </c>
-      <c r="K48" s="17" t="n"/>
+      <c r="K48" s="17" t="n">
+        <v>12</v>
+      </c>
       <c r="L48" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M48" s="3" t="inlineStr">
         <is>
@@ -4810,14 +4843,20 @@
       <c r="O48" s="19" t="n">
         <v>46246</v>
       </c>
-      <c r="P48" s="3" t="n"/>
+      <c r="P48" s="19" t="n">
+        <v>46239</v>
+      </c>
       <c r="Q48" s="3" t="inlineStr">
         <is>
           <t>Unauthorized callers receive 403 on sensitive routes</t>
         </is>
       </c>
       <c r="R48" s="3" t="inlineStr"/>
-      <c r="S48" s="3" t="inlineStr"/>
+      <c r="S48" s="3" t="inlineStr">
+        <is>
+          <t>require_admin_if_auth on credentials/settings/models/embedding_rebuild</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="75" customHeight="1">
       <c r="A49" s="3" t="inlineStr">
@@ -4847,9 +4886,9 @@
           <t>Schema + query ownership filters</t>
         </is>
       </c>
-      <c r="F49" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F49" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G49" s="20" t="inlineStr">
@@ -4868,9 +4907,11 @@
       <c r="J49" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="K49" s="17" t="n"/>
+      <c r="K49" s="17" t="n">
+        <v>24</v>
+      </c>
       <c r="L49" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M49" s="3" t="inlineStr">
         <is>
@@ -4883,7 +4924,9 @@
       <c r="O49" s="19" t="n">
         <v>46249</v>
       </c>
-      <c r="P49" s="3" t="n"/>
+      <c r="P49" s="19" t="n">
+        <v>46239</v>
+      </c>
       <c r="Q49" s="3" t="inlineStr">
         <is>
           <t>Users only see their own notebooks/sources</t>
@@ -4894,7 +4937,11 @@
           <t>Highest-risk WP2 task</t>
         </is>
       </c>
-      <c r="S49" s="3" t="inlineStr"/>
+      <c r="S49" s="3" t="inlineStr">
+        <is>
+          <t>ownership filters notebooks/sources/notes/chat/podcasts/search</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="75" customHeight="1">
       <c r="A50" s="3" t="inlineStr">
@@ -4923,9 +4970,9 @@
           <t>Entra login UX + session handling</t>
         </is>
       </c>
-      <c r="F50" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F50" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G50" s="20" t="inlineStr">
@@ -4944,9 +4991,11 @@
       <c r="J50" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="K50" s="17" t="n"/>
+      <c r="K50" s="17" t="n">
+        <v>24</v>
+      </c>
       <c r="L50" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M50" s="3" t="inlineStr">
         <is>
@@ -4959,14 +5008,20 @@
       <c r="O50" s="19" t="n">
         <v>46247</v>
       </c>
-      <c r="P50" s="3" t="n"/>
+      <c r="P50" s="19" t="n">
+        <v>46239</v>
+      </c>
       <c r="Q50" s="3" t="inlineStr">
         <is>
           <t>Login via a real Entra account works end-to-end</t>
         </is>
       </c>
       <c r="R50" s="3" t="inlineStr"/>
-      <c r="S50" s="3" t="inlineStr"/>
+      <c r="S50" s="3" t="inlineStr">
+        <is>
+          <t>Entra LoginForm + auth-store cookie session</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="75" customHeight="1">
       <c r="A51" s="3" t="inlineStr">
@@ -4995,9 +5050,9 @@
           <t>GenericOIDCProvider stub + test</t>
         </is>
       </c>
-      <c r="F51" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F51" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G51" s="21" t="inlineStr">
@@ -5016,9 +5071,11 @@
       <c r="J51" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="K51" s="17" t="n"/>
+      <c r="K51" s="17" t="n">
+        <v>8</v>
+      </c>
       <c r="L51" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M51" s="3" t="inlineStr">
         <is>
@@ -5031,14 +5088,20 @@
       <c r="O51" s="19" t="n">
         <v>46248</v>
       </c>
-      <c r="P51" s="3" t="n"/>
+      <c r="P51" s="19" t="n">
+        <v>46239</v>
+      </c>
       <c r="Q51" s="3" t="inlineStr">
         <is>
           <t>Adding a second provider requires no change to route handlers</t>
         </is>
       </c>
       <c r="R51" s="3" t="inlineStr"/>
-      <c r="S51" s="3" t="inlineStr"/>
+      <c r="S51" s="3" t="inlineStr">
+        <is>
+          <t>pluggability tests without route coupling</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="75" customHeight="1">
       <c r="A52" s="3" t="inlineStr">
@@ -5067,9 +5130,9 @@
           <t>docs/AUTH.md</t>
         </is>
       </c>
-      <c r="F52" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F52" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G52" s="16" t="inlineStr">
@@ -5088,9 +5151,11 @@
       <c r="J52" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="K52" s="17" t="n"/>
+      <c r="K52" s="17" t="n">
+        <v>8</v>
+      </c>
       <c r="L52" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M52" s="3" t="inlineStr">
         <is>
@@ -5103,14 +5168,20 @@
       <c r="O52" s="19" t="n">
         <v>46249</v>
       </c>
-      <c r="P52" s="3" t="n"/>
+      <c r="P52" s="19" t="n">
+        <v>46239</v>
+      </c>
       <c r="Q52" s="3" t="inlineStr">
         <is>
           <t>AUTH.md complete for operators</t>
         </is>
       </c>
       <c r="R52" s="3" t="inlineStr"/>
-      <c r="S52" s="3" t="inlineStr"/>
+      <c r="S52" s="3" t="inlineStr">
+        <is>
+          <t>docs/AUTH.md</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="75" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
@@ -5139,9 +5210,9 @@
           <t>Green PR wp-2-entra-auth</t>
         </is>
       </c>
-      <c r="F53" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F53" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G53" s="20" t="inlineStr">
@@ -5160,9 +5231,11 @@
       <c r="J53" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="K53" s="17" t="n"/>
+      <c r="K53" s="17" t="n">
+        <v>16</v>
+      </c>
       <c r="L53" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M53" s="3" t="inlineStr">
         <is>
@@ -5175,358 +5248,408 @@
       <c r="O53" s="19" t="n">
         <v>46252</v>
       </c>
-      <c r="P53" s="3" t="n"/>
+      <c r="P53" s="19" t="n">
+        <v>46239</v>
+      </c>
       <c r="Q53" s="3" t="inlineStr">
         <is>
-          <t>All WP2 acceptance criteria pass; CI green</t>
+          <t>All WP2 acceptance criteria pass; PR merged to HariHaranDFX/open-notebook main</t>
         </is>
       </c>
       <c r="R53" s="3" t="inlineStr">
         <is>
-          <t>Largest single change in the program</t>
-        </is>
-      </c>
-      <c r="S53" s="3" t="inlineStr"/>
+          <t>Human review stop after merge; do not start WP3 on same branch</t>
+        </is>
+      </c>
+      <c r="S53" s="3" t="inlineStr">
+        <is>
+          <t>PR wp-2-entra-auth</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="75" customHeight="1">
       <c r="A54" s="3" t="inlineStr">
         <is>
+          <t>4.11</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>WP2 — Identity &amp; Entra Auth</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Transformation ownership (shared/personal + soft-delete builtins)</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: stop any user from deleting/editing the shared transformation catalog for everyone.
+Steps: migration 27 (user_id, is_builtin, deleted_at); builtins soft-delete + admin restore; admin-created shared hard-delete; user-created personal CRUD; restore Analyze Paper; frontend badges/restore + filter archived from pickers.</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>transformation_access + migration 27</t>
+        </is>
+      </c>
+      <c r="F54" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G54" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>4.5,4.6</t>
+        </is>
+      </c>
+      <c r="I54" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="J54" s="17" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K54" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="L54" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M54" s="3" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="N54" s="19" t="n">
+        <v>46239</v>
+      </c>
+      <c r="O54" s="19" t="n">
+        <v>46239</v>
+      </c>
+      <c r="P54" s="19" t="n">
+        <v>46239</v>
+      </c>
+      <c r="Q54" s="3" t="inlineStr">
+        <is>
+          <t>Shared catalog admin-only mutate; personal owner-only; builtins restorable</t>
+        </is>
+      </c>
+      <c r="R54" s="3" t="inlineStr">
+        <is>
+          <t>Follow-on discovered during WP2 Entra testing</t>
+        </is>
+      </c>
+      <c r="S54" s="3" t="inlineStr">
+        <is>
+          <t>api/transformation_access.py; migrations/27.surrealql</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="75" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>4.12</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>WP2 — Identity &amp; Entra Auth</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Meaningful permission error messages (API + UI)</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: replace generic Error / Not allowed toasts when non-admins hit forbidden actions.
+Steps: specific 403 details for transformation edit/delete/restore and admin gates; ERROR_MAP + i18n; 403 safety net; fix getApiErrorKey misuse; gate default-prompt PUT to admin.</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>error-handler + transformation_access messages</t>
+        </is>
+      </c>
+      <c r="F55" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G55" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>4.5,4.11</t>
+        </is>
+      </c>
+      <c r="I55" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="J55" s="17" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K55" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="L55" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M55" s="3" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="N55" s="19" t="n">
+        <v>46239</v>
+      </c>
+      <c r="O55" s="19" t="n">
+        <v>46239</v>
+      </c>
+      <c r="P55" s="19" t="n">
+        <v>46239</v>
+      </c>
+      <c r="Q55" s="3" t="inlineStr">
+        <is>
+          <t>Forbidden actions show clear admin/owner messages, never bare Error</t>
+        </is>
+      </c>
+      <c r="R55" s="3" t="inlineStr">
+        <is>
+          <t>Additional UX hardening during WP2</t>
+        </is>
+      </c>
+      <c r="S55" s="3" t="inlineStr">
+        <is>
+          <t>frontend/src/lib/utils/error-handler.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="75" customHeight="1">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>4.13</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>WP2 — Identity &amp; Entra Auth</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Admin-only UI gating (nav + routes)</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: hide Models/Settings/Advanced (and related surfaces) from normal users; show only to admins.
+Steps: persist role from /auth/me; isAdmin helper; filter sidebar + command palette; AdminOnly route guard; hide SetupBanner + default prompt editor for non-admins.</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>AdminOnly + auth role in store</t>
+        </is>
+      </c>
+      <c r="F56" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G56" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>4.5,4.7</t>
+        </is>
+      </c>
+      <c r="I56" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="J56" s="17" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K56" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="L56" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M56" s="3" t="inlineStr">
+        <is>
+          <t>Frontend Engineer</t>
+        </is>
+      </c>
+      <c r="N56" s="19" t="n">
+        <v>46239</v>
+      </c>
+      <c r="O56" s="19" t="n">
+        <v>46239</v>
+      </c>
+      <c r="P56" s="19" t="n">
+        <v>46239</v>
+      </c>
+      <c r="Q56" s="3" t="inlineStr">
+        <is>
+          <t>Non-admin never sees admin nav; direct URL redirects to notebooks</t>
+        </is>
+      </c>
+      <c r="R56" s="3" t="inlineStr">
+        <is>
+          <t>UI companion to API admin gates</t>
+        </is>
+      </c>
+      <c r="S56" s="3" t="inlineStr">
+        <is>
+          <t>frontend/src/components/auth/AdminOnly.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="75" customHeight="1">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>4.14</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>WP2 — Identity &amp; Entra Auth</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Sidebar active-state longest-prefix fix</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: fix Models (/settings/api-keys) also highlighting Settings (/settings).
+Steps: replace pathname.startsWith(href) with longest matching nav href wins.</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>nav-active helper</t>
+        </is>
+      </c>
+      <c r="F57" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G57" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>4.13</t>
+        </is>
+      </c>
+      <c r="I57" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J57" s="17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K57" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L57" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M57" s="3" t="inlineStr">
+        <is>
+          <t>Frontend Engineer</t>
+        </is>
+      </c>
+      <c r="N57" s="19" t="n">
+        <v>46239</v>
+      </c>
+      <c r="O57" s="19" t="n">
+        <v>46239</v>
+      </c>
+      <c r="P57" s="19" t="n">
+        <v>46239</v>
+      </c>
+      <c r="Q57" s="3" t="inlineStr">
+        <is>
+          <t>Only Models active on /settings/api-keys</t>
+        </is>
+      </c>
+      <c r="R57" s="3" t="inlineStr">
+        <is>
+          <t>Bug found during WP2 UI verification</t>
+        </is>
+      </c>
+      <c r="S57" s="3" t="inlineStr">
+        <is>
+          <t>frontend/src/components/layout/nav-active.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="75" customHeight="1">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
           <t>5.0</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>WP3 — Frontend Map + White-label</t>
         </is>
       </c>
-      <c r="C54" s="3" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>WP3 kickoff</t>
         </is>
       </c>
-      <c r="D54" s="3" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>Purpose: start white-label work only after identity is on main.
 Steps: create wp-3-white-label; confirm Model A brand loads once at app startup (not per request).</t>
         </is>
       </c>
-      <c r="E54" s="3" t="inlineStr">
+      <c r="E58" s="3" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="F54" s="22" t="inlineStr">
+      <c r="F58" s="22" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G54" s="16" t="inlineStr">
+      <c r="G58" s="16" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H54" s="3" t="inlineStr">
+      <c r="H58" s="3" t="inlineStr">
         <is>
           <t>4.10</t>
         </is>
       </c>
-      <c r="I54" s="17" t="n">
+      <c r="I58" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="J54" s="17" t="n">
+      <c r="J58" s="17" t="n">
         <v>0.25</v>
-      </c>
-      <c r="K54" s="17" t="n"/>
-      <c r="L54" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M54" s="3" t="inlineStr">
-        <is>
-          <t>Frontend Engineer</t>
-        </is>
-      </c>
-      <c r="N54" s="19" t="n">
-        <v>46253</v>
-      </c>
-      <c r="O54" s="19" t="n">
-        <v>46253</v>
-      </c>
-      <c r="P54" s="3" t="n"/>
-      <c r="Q54" s="3" t="inlineStr">
-        <is>
-          <t>Branch created after WP2 merge</t>
-        </is>
-      </c>
-      <c r="R54" s="3" t="inlineStr">
-        <is>
-          <t>Optional admin brand UI needs WP2 roles</t>
-        </is>
-      </c>
-      <c r="S54" s="3" t="inlineStr"/>
-    </row>
-    <row r="55" ht="75" customHeight="1">
-      <c r="A55" s="3" t="inlineStr">
-        <is>
-          <t>5.1</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>WP3 — Frontend Map + White-label</t>
-        </is>
-      </c>
-      <c r="C55" s="3" t="inlineStr">
-        <is>
-          <t>Produce docs/FRONTEND_MAP.md</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>Purpose: make every future UI change locatable without archaeology.
-Steps: for each auth and dashboard route, document page → component tree, stores/hooks/API calls, shared layout, component catalog, and a where-do-I-change-X table.</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>docs/FRONTEND_MAP.md</t>
-        </is>
-      </c>
-      <c r="F55" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G55" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H55" s="3" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="I55" s="17" t="n">
-        <v>20</v>
-      </c>
-      <c r="J55" s="17" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="K55" s="17" t="n"/>
-      <c r="L55" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M55" s="3" t="inlineStr">
-        <is>
-          <t>Frontend Engineer</t>
-        </is>
-      </c>
-      <c r="N55" s="19" t="n">
-        <v>46253</v>
-      </c>
-      <c r="O55" s="19" t="n">
-        <v>46255</v>
-      </c>
-      <c r="P55" s="3" t="n"/>
-      <c r="Q55" s="3" t="inlineStr">
-        <is>
-          <t>Map covers every route with data flow + backend calls</t>
-        </is>
-      </c>
-      <c r="R55" s="3" t="inlineStr"/>
-      <c r="S55" s="3" t="inlineStr"/>
-    </row>
-    <row r="56" ht="75" customHeight="1">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>5.2</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>WP3 — Frontend Map + White-label</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>BrandConfig schema + loader</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>Purpose: drive app name, logos, favicon, colours, font, and support URL from config so clients do not need a rebuild.
-Steps: define BrandConfig schema; load from BRAND_CONFIG_PATH or /config/brand at startup under Model A.</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>BrandConfig type + loader</t>
-        </is>
-      </c>
-      <c r="F56" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G56" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H56" s="3" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="I56" s="17" t="n">
-        <v>12</v>
-      </c>
-      <c r="J56" s="17" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="K56" s="17" t="n"/>
-      <c r="L56" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M56" s="3" t="inlineStr">
-        <is>
-          <t>Full-stack</t>
-        </is>
-      </c>
-      <c r="N56" s="19" t="n">
-        <v>46255</v>
-      </c>
-      <c r="O56" s="19" t="n">
-        <v>46256</v>
-      </c>
-      <c r="P56" s="3" t="n"/>
-      <c r="Q56" s="3" t="inlineStr">
-        <is>
-          <t>Config loads without a rebuild</t>
-        </is>
-      </c>
-      <c r="R56" s="3" t="inlineStr"/>
-      <c r="S56" s="3" t="inlineStr"/>
-    </row>
-    <row r="57" ht="75" customHeight="1">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>5.3</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>WP3 — Frontend Map + White-label</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>Runtime theme injection (CSS variables)</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>Purpose: apply BrandConfig at runtime to CSS variables for light and dark themes.
-Steps: map colours to :root / dark variants; replace hardcoded title and /logo.svg; use the brand inventory in LICENSE_COMPLIANCE §8; demonstrate two brands from one build.</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>Runtime theming</t>
-        </is>
-      </c>
-      <c r="F57" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G57" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H57" s="3" t="inlineStr">
-        <is>
-          <t>5.2</t>
-        </is>
-      </c>
-      <c r="I57" s="17" t="n">
-        <v>16</v>
-      </c>
-      <c r="J57" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="K57" s="17" t="n"/>
-      <c r="L57" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M57" s="3" t="inlineStr">
-        <is>
-          <t>Frontend Engineer</t>
-        </is>
-      </c>
-      <c r="N57" s="19" t="n">
-        <v>46256</v>
-      </c>
-      <c r="O57" s="19" t="n">
-        <v>46259</v>
-      </c>
-      <c r="P57" s="3" t="n"/>
-      <c r="Q57" s="3" t="inlineStr">
-        <is>
-          <t>Two visibly different brands from the same build; no code edit to rebrand</t>
-        </is>
-      </c>
-      <c r="R57" s="3" t="inlineStr"/>
-      <c r="S57" s="3" t="inlineStr"/>
-    </row>
-    <row r="58" ht="75" customHeight="1">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>5.4</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>WP3 — Frontend Map + White-label</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>themes/ presets + add-client procedure</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>Purpose: make “add a client theme” a documented drop-in of config + assets.
-Steps: ship at least two presets under themes/; write the operator procedure (no rebuild).</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr">
-        <is>
-          <t>themes/ + docs procedure</t>
-        </is>
-      </c>
-      <c r="F58" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G58" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H58" s="3" t="inlineStr">
-        <is>
-          <t>5.3</t>
-        </is>
-      </c>
-      <c r="I58" s="17" t="n">
-        <v>8</v>
-      </c>
-      <c r="J58" s="17" t="n">
-        <v>1</v>
       </c>
       <c r="K58" s="17" t="n"/>
       <c r="L58" s="18" t="n">
@@ -5538,24 +5661,28 @@
         </is>
       </c>
       <c r="N58" s="19" t="n">
-        <v>46259</v>
+        <v>46253</v>
       </c>
       <c r="O58" s="19" t="n">
-        <v>46260</v>
+        <v>46253</v>
       </c>
       <c r="P58" s="3" t="n"/>
       <c r="Q58" s="3" t="inlineStr">
         <is>
-          <t>Documented procedure produces two different brands from one build</t>
-        </is>
-      </c>
-      <c r="R58" s="3" t="inlineStr"/>
+          <t>Branch created after WP2 merge</t>
+        </is>
+      </c>
+      <c r="R58" s="3" t="inlineStr">
+        <is>
+          <t>Optional admin brand UI needs WP2 roles</t>
+        </is>
+      </c>
       <c r="S58" s="3" t="inlineStr"/>
     </row>
     <row r="59" ht="75" customHeight="1">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -5565,18 +5692,18 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Optional admin BrandConfig UI</t>
+          <t>Produce docs/FRONTEND_MAP.md</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Purpose (optional): let admins edit BrandConfig live without redeploying.
-Steps: admin-only settings screen gated by WP2 roles; persist and hot-apply theme.</t>
+          <t>Purpose: make every future UI change locatable without archaeology.
+Steps: for each auth and dashboard route, document page → component tree, stores/hooks/API calls, shared layout, component catalog, and a where-do-I-change-X table.</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Admin brand settings UI</t>
+          <t>docs/FRONTEND_MAP.md</t>
         </is>
       </c>
       <c r="F59" s="22" t="inlineStr">
@@ -5584,21 +5711,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G59" s="24" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="G59" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>5.3,4.5</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="I59" s="17" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="J59" s="17" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="K59" s="17" t="n"/>
       <c r="L59" s="18" t="n">
@@ -5610,28 +5737,24 @@
         </is>
       </c>
       <c r="N59" s="19" t="n">
-        <v>46260</v>
+        <v>46253</v>
       </c>
       <c r="O59" s="19" t="n">
-        <v>46262</v>
+        <v>46255</v>
       </c>
       <c r="P59" s="3" t="n"/>
       <c r="Q59" s="3" t="inlineStr">
         <is>
-          <t>Admin can edit brand without redeploy (optional acceptance)</t>
-        </is>
-      </c>
-      <c r="R59" s="3" t="inlineStr">
-        <is>
-          <t>Optional per master plan</t>
-        </is>
-      </c>
+          <t>Map covers every route with data flow + backend calls</t>
+        </is>
+      </c>
+      <c r="R59" s="3" t="inlineStr"/>
       <c r="S59" s="3" t="inlineStr"/>
     </row>
     <row r="60" ht="75" customHeight="1">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>5.2</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -5641,18 +5764,18 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>WP3 verification + review stop</t>
+          <t>BrandConfig schema + loader</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Purpose: close white-label only when map + config branding acceptance criteria pass.
-Steps: verify ACs; PR; human review; do not mix WP5 on the same branch.</t>
+          <t>Purpose: drive app name, logos, favicon, colours, font, and support URL from config so clients do not need a rebuild.
+Steps: define BrandConfig schema; load from BRAND_CONFIG_PATH or /config/brand at startup under Model A.</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Merged WP3</t>
+          <t>BrandConfig type + loader</t>
         </is>
       </c>
       <c r="F60" s="22" t="inlineStr">
@@ -5660,21 +5783,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G60" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G60" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>5.1,5.4</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="I60" s="17" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J60" s="17" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="K60" s="17" t="n"/>
       <c r="L60" s="18" t="n">
@@ -5682,19 +5805,19 @@
       </c>
       <c r="M60" s="3" t="inlineStr">
         <is>
-          <t>Engineering Lead</t>
+          <t>Full-stack</t>
         </is>
       </c>
       <c r="N60" s="19" t="n">
-        <v>46262</v>
+        <v>46255</v>
       </c>
       <c r="O60" s="19" t="n">
-        <v>46263</v>
+        <v>46256</v>
       </c>
       <c r="P60" s="3" t="n"/>
       <c r="Q60" s="3" t="inlineStr">
         <is>
-          <t>All WP3 acceptance criteria pass</t>
+          <t>Config loads without a rebuild</t>
         </is>
       </c>
       <c r="R60" s="3" t="inlineStr"/>
@@ -5703,28 +5826,28 @@
     <row r="61" ht="75" customHeight="1">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>WP4 — Backend/API Documentation</t>
+          <t>WP3 — Frontend Map + White-label</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>WP4 kickoff (can parallel early)</t>
+          <t>Runtime theme injection (CSS variables)</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Purpose: start the backend architecture map as documentation-only, low-risk work.
-Steps: create wp-4-backend-map; prefer starting after WP2 so auth docs match reality; can begin after WP0 if staffed in parallel.</t>
+          <t>Purpose: apply BrandConfig at runtime to CSS variables for light and dark themes.
+Steps: map colours to :root / dark variants; replace hardcoded title and /logo.svg; use the brand inventory in LICENSE_COMPLIANCE §8; demonstrate two brands from one build.</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>Runtime theming</t>
         </is>
       </c>
       <c r="F61" s="22" t="inlineStr">
@@ -5732,21 +5855,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G61" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G61" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>5.2</t>
         </is>
       </c>
       <c r="I61" s="17" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="J61" s="17" t="n">
-        <v>0.25</v>
+        <v>2</v>
       </c>
       <c r="K61" s="17" t="n"/>
       <c r="L61" s="18" t="n">
@@ -5754,53 +5877,49 @@
       </c>
       <c r="M61" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N61" s="19" t="n">
-        <v>46253</v>
+        <v>46256</v>
       </c>
       <c r="O61" s="19" t="n">
-        <v>46253</v>
+        <v>46259</v>
       </c>
       <c r="P61" s="3" t="n"/>
       <c r="Q61" s="3" t="inlineStr">
         <is>
-          <t>Docs branch ready</t>
-        </is>
-      </c>
-      <c r="R61" s="3" t="inlineStr">
-        <is>
-          <t>Better after WP2 for accurate auth sections</t>
-        </is>
-      </c>
+          <t>Two visibly different brands from the same build; no code edit to rebrand</t>
+        </is>
+      </c>
+      <c r="R61" s="3" t="inlineStr"/>
       <c r="S61" s="3" t="inlineStr"/>
     </row>
     <row r="62" ht="75" customHeight="1">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>WP4 — Backend/API Documentation</t>
+          <t>WP3 — Frontend Map + White-label</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Router catalog (all endpoints)</t>
+          <t>themes/ presets + add-client procedure</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Purpose: catalogue every HTTP endpoint with method, path, models, auth requirement, and service/domain call.
-Steps: walk all routers; document consistently; update after WP2 auth lands.</t>
+          <t>Purpose: make “add a client theme” a documented drop-in of config + assets.
+Steps: ship at least two presets under themes/; write the operator procedure (no rebuild).</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>BACKEND_MAP.md routers section</t>
+          <t>themes/ + docs procedure</t>
         </is>
       </c>
       <c r="F62" s="22" t="inlineStr">
@@ -5808,21 +5927,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G62" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G62" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="I62" s="17" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="J62" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K62" s="17" t="n"/>
       <c r="L62" s="18" t="n">
@@ -5830,19 +5949,19 @@
       </c>
       <c r="M62" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N62" s="19" t="n">
-        <v>46253</v>
+        <v>46259</v>
       </c>
       <c r="O62" s="19" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="P62" s="3" t="n"/>
       <c r="Q62" s="3" t="inlineStr">
         <is>
-          <t>Every endpoint documented with auth + models</t>
+          <t>Documented procedure produces two different brands from one build</t>
         </is>
       </c>
       <c r="R62" s="3" t="inlineStr"/>
@@ -5851,28 +5970,28 @@
     <row r="63" ht="75" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>WP4 — Backend/API Documentation</t>
+          <t>WP3 — Frontend Map + White-label</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Domain model + graph + data layer maps</t>
+          <t>Optional admin BrandConfig UI</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Purpose: document ObjectModel patterns, LangGraph flows, repository usage, migrations, and SurrealDB features in use.
-Steps: catalogue models/relationships; map each graph’s inputs/steps/outputs; explain repository call-site pattern and migrations.</t>
+          <t>Purpose (optional): let admins edit BrandConfig live without redeploying.
+Steps: admin-only settings screen gated by WP2 roles; persist and hot-apply theme.</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>BACKEND_MAP.md domain/graphs/data</t>
+          <t>Admin brand settings UI</t>
         </is>
       </c>
       <c r="F63" s="22" t="inlineStr">
@@ -5880,14 +5999,14 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G63" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G63" s="24" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.3,4.5</t>
         </is>
       </c>
       <c r="I63" s="17" t="n">
@@ -5902,49 +6021,53 @@
       </c>
       <c r="M63" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N63" s="19" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="O63" s="19" t="n">
-        <v>46259</v>
+        <v>46262</v>
       </c>
       <c r="P63" s="3" t="n"/>
       <c r="Q63" s="3" t="inlineStr">
         <is>
-          <t>Every domain model and graph documented</t>
-        </is>
-      </c>
-      <c r="R63" s="3" t="inlineStr"/>
+          <t>Admin can edit brand without redeploy (optional acceptance)</t>
+        </is>
+      </c>
+      <c r="R63" s="3" t="inlineStr">
+        <is>
+          <t>Optional per master plan</t>
+        </is>
+      </c>
       <c r="S63" s="3" t="inlineStr"/>
     </row>
     <row r="64" ht="75" customHeight="1">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>6.3</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>WP4 — Backend/API Documentation</t>
+          <t>WP3 — Frontend Map + White-label</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Jobs, config/secrets, how-to playbooks</t>
+          <t>WP3 verification + review stop</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Purpose: finish the operator/engineer map with jobs, env vars, and five how-to-add playbooks.
-Steps: document surreal-commands; env/secrets; playbooks for endpoint, model+migration, provider, job, source type; reconcile with existing change-playbooks.md.</t>
+          <t>Purpose: close white-label only when map + config branding acceptance criteria pass.
+Steps: verify ACs; PR; human review; do not mix WP5 on the same branch.</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>BACKEND_MAP.md complete</t>
+          <t>Merged WP3</t>
         </is>
       </c>
       <c r="F64" s="22" t="inlineStr">
@@ -5952,21 +6075,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G64" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G64" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>5.1,5.4</t>
         </is>
       </c>
       <c r="I64" s="17" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="J64" s="17" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="K64" s="17" t="n"/>
       <c r="L64" s="18" t="n">
@@ -5974,19 +6097,19 @@
       </c>
       <c r="M64" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Engineering Lead</t>
         </is>
       </c>
       <c r="N64" s="19" t="n">
-        <v>46259</v>
+        <v>46262</v>
       </c>
       <c r="O64" s="19" t="n">
-        <v>46260</v>
+        <v>46263</v>
       </c>
       <c r="P64" s="3" t="n"/>
       <c r="Q64" s="3" t="inlineStr">
         <is>
-          <t>Five how-to playbooks present and accurate</t>
+          <t>All WP3 acceptance criteria pass</t>
         </is>
       </c>
       <c r="R64" s="3" t="inlineStr"/>
@@ -5995,7 +6118,7 @@
     <row r="65" ht="75" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>6.4</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -6005,18 +6128,18 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>WP4 review stop</t>
+          <t>WP4 kickoff (can parallel early)</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Purpose: peer-review the map for accuracy and merge.
-Steps: review against live code; fix gaps; merge; confirm a new engineer can locate changes using only BACKEND_MAP.</t>
+          <t>Purpose: start the backend architecture map as documentation-only, low-risk work.
+Steps: create wp-4-backend-map; prefer starting after WP2 so auth docs match reality; can begin after WP0 if staffed in parallel.</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>docs/BACKEND_MAP.md on main</t>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F65" s="22" t="inlineStr">
@@ -6031,14 +6154,14 @@
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>6.3</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="I65" s="17" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J65" s="17" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="K65" s="17" t="n"/>
       <c r="L65" s="18" t="n">
@@ -6046,49 +6169,53 @@
       </c>
       <c r="M65" s="3" t="inlineStr">
         <is>
-          <t>Engineering Lead</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N65" s="19" t="n">
-        <v>46260</v>
+        <v>46253</v>
       </c>
       <c r="O65" s="19" t="n">
-        <v>46261</v>
+        <v>46253</v>
       </c>
       <c r="P65" s="3" t="n"/>
       <c r="Q65" s="3" t="inlineStr">
         <is>
-          <t>New engineer can locate changes using only this doc</t>
-        </is>
-      </c>
-      <c r="R65" s="3" t="inlineStr"/>
+          <t>Docs branch ready</t>
+        </is>
+      </c>
+      <c r="R65" s="3" t="inlineStr">
+        <is>
+          <t>Better after WP2 for accurate auth sections</t>
+        </is>
+      </c>
       <c r="S65" s="3" t="inlineStr"/>
     </row>
     <row r="66" ht="75" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>7.0</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>WP5 — External Source Connectors</t>
+          <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>WP5 kickoff</t>
+          <t>Router catalog (all endpoints)</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Purpose: design connectors that feed the existing ingestion pipeline instead of reinventing extraction.
-Steps: create wp-5-connectors; draft SourceConnector interface; confirm hard dependency on WP2 for per-user OAuth tokens.</t>
+          <t>Purpose: catalogue every HTTP endpoint with method, path, models, auth requirement, and service/domain call.
+Steps: walk all routers; document consistently; update after WP2 auth lands.</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Branch + design note</t>
+          <t>BACKEND_MAP.md routers section</t>
         </is>
       </c>
       <c r="F66" s="22" t="inlineStr">
@@ -6096,21 +6223,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G66" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G66" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>4.10</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="I66" s="17" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="J66" s="17" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="K66" s="17" t="n"/>
       <c r="L66" s="18" t="n">
@@ -6118,53 +6245,49 @@
       </c>
       <c r="M66" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N66" s="19" t="n">
-        <v>46266</v>
+        <v>46253</v>
       </c>
       <c r="O66" s="19" t="n">
-        <v>46266</v>
+        <v>46255</v>
       </c>
       <c r="P66" s="3" t="n"/>
       <c r="Q66" s="3" t="inlineStr">
         <is>
-          <t>Design reuses content-core + graphs/source.py</t>
-        </is>
-      </c>
-      <c r="R66" s="3" t="inlineStr">
-        <is>
-          <t>Blocked until WP2 users/tokens exist</t>
-        </is>
-      </c>
+          <t>Every endpoint documented with auth + models</t>
+        </is>
+      </c>
+      <c r="R66" s="3" t="inlineStr"/>
       <c r="S66" s="3" t="inlineStr"/>
     </row>
     <row r="67" ht="75" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>WP5 — External Source Connectors</t>
+          <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>SourceConnector interface + bulk job fan-out</t>
+          <t>Domain model + graph + data layer maps</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Purpose: one “add location” action becomes N document jobs with per-doc progress and partial failure tolerance.
-Steps: define authenticate/list_documents/fetch_document; extend source_commands for fan-out; ensure one bad file does not abort the batch.</t>
+          <t>Purpose: document ObjectModel patterns, LangGraph flows, repository usage, migrations, and SurrealDB features in use.
+Steps: catalogue models/relationships; map each graph’s inputs/steps/outputs; explain repository call-site pattern and migrations.</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Connector API + bulk command</t>
+          <t>BACKEND_MAP.md domain/graphs/data</t>
         </is>
       </c>
       <c r="F67" s="22" t="inlineStr">
@@ -6172,21 +6295,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G67" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G67" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>7.0</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="I67" s="17" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="J67" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K67" s="17" t="n"/>
       <c r="L67" s="18" t="n">
@@ -6198,15 +6321,15 @@
         </is>
       </c>
       <c r="N67" s="19" t="n">
-        <v>46266</v>
+        <v>46255</v>
       </c>
       <c r="O67" s="19" t="n">
-        <v>46269</v>
+        <v>46259</v>
       </c>
       <c r="P67" s="3" t="n"/>
       <c r="Q67" s="3" t="inlineStr">
         <is>
-          <t>Single failure does not abort batch; progress per document</t>
+          <t>Every domain model and graph documented</t>
         </is>
       </c>
       <c r="R67" s="3" t="inlineStr"/>
@@ -6215,28 +6338,28 @@
     <row r="68" ht="75" customHeight="1">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>6.3</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>WP5 — External Source Connectors</t>
+          <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>SharePoint connector (Microsoft Graph)</t>
+          <t>Jobs, config/secrets, how-to playbooks</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Purpose: let an Entra-signed-in user pull an entire SharePoint folder into chat-able sources.
-Steps: OAuth on behalf of the user; least-privilege Sites/Files read scopes; enumerate folder; download supported files into existing ingestion; document admin consent.</t>
+          <t>Purpose: finish the operator/engineer map with jobs, env vars, and five how-to-add playbooks.
+Steps: document surreal-commands; env/secrets; playbooks for endpoint, model+migration, provider, job, source type; reconcile with existing change-playbooks.md.</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>SharePointConnector</t>
+          <t>BACKEND_MAP.md complete</t>
         </is>
       </c>
       <c r="F68" s="22" t="inlineStr">
@@ -6244,21 +6367,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G68" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G68" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>7.1,4.7</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="I68" s="17" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="J68" s="17" t="n">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="K68" s="17" t="n"/>
       <c r="L68" s="18" t="n">
@@ -6270,15 +6393,15 @@
         </is>
       </c>
       <c r="N68" s="19" t="n">
-        <v>46269</v>
+        <v>46259</v>
       </c>
       <c r="O68" s="19" t="n">
-        <v>46275</v>
+        <v>46260</v>
       </c>
       <c r="P68" s="3" t="n"/>
       <c r="Q68" s="3" t="inlineStr">
         <is>
-          <t>User connects SharePoint, picks folder, pulls all supported docs</t>
+          <t>Five how-to playbooks present and accurate</t>
         </is>
       </c>
       <c r="R68" s="3" t="inlineStr"/>
@@ -6287,28 +6410,28 @@
     <row r="69" ht="75" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>WP5 — External Source Connectors</t>
+          <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Generic DMS / multi-doc link connector</t>
+          <t>WP4 review stop</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Purpose: support folder URLs / IDs that resolve to many documents, with an extension point for other DMS systems.
-Steps: implement base multi-doc connector; keep the SourceConnector interface as the only required surface for new connectors.</t>
+          <t>Purpose: peer-review the map for accuracy and merge.
+Steps: review against live code; fix gaps; merge; confirm a new engineer can locate changes using only BACKEND_MAP.</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Generic multi-doc connector</t>
+          <t>docs/BACKEND_MAP.md on main</t>
         </is>
       </c>
       <c r="F69" s="22" t="inlineStr">
@@ -6316,21 +6439,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G69" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G69" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.3</t>
         </is>
       </c>
       <c r="I69" s="17" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="J69" s="17" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="K69" s="17" t="n"/>
       <c r="L69" s="18" t="n">
@@ -6338,19 +6461,19 @@
       </c>
       <c r="M69" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Engineering Lead</t>
         </is>
       </c>
       <c r="N69" s="19" t="n">
-        <v>46273</v>
+        <v>46260</v>
       </c>
       <c r="O69" s="19" t="n">
-        <v>46275</v>
+        <v>46261</v>
       </c>
       <c r="P69" s="3" t="n"/>
       <c r="Q69" s="3" t="inlineStr">
         <is>
-          <t>New connector = implement interface only</t>
+          <t>New engineer can locate changes using only this doc</t>
         </is>
       </c>
       <c r="R69" s="3" t="inlineStr"/>
@@ -6359,7 +6482,7 @@
     <row r="70" ht="75" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>7.4</t>
+          <t>7.0</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -6369,18 +6492,18 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Encrypted per-user token storage</t>
+          <t>WP5 kickoff</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Purpose: store connector OAuth tokens encrypted per user using existing encryption-key infrastructure.
-Steps: persist tokens encrypted; never share across users; respect source-system permissions (never fetch what the user cannot access).</t>
+          <t>Purpose: design connectors that feed the existing ingestion pipeline instead of reinventing extraction.
+Steps: create wp-5-connectors; draft SourceConnector interface; confirm hard dependency on WP2 for per-user OAuth tokens.</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Encrypted token store</t>
+          <t>Branch + design note</t>
         </is>
       </c>
       <c r="F70" s="22" t="inlineStr">
@@ -6388,21 +6511,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G70" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G70" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>7.2,2.8</t>
+          <t>4.10</t>
         </is>
       </c>
       <c r="I70" s="17" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="J70" s="17" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="K70" s="17" t="n"/>
       <c r="L70" s="18" t="n">
@@ -6410,28 +6533,32 @@
       </c>
       <c r="M70" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N70" s="19" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="O70" s="19" t="n">
-        <v>46276</v>
+        <v>46266</v>
       </c>
       <c r="P70" s="3" t="n"/>
       <c r="Q70" s="3" t="inlineStr">
         <is>
-          <t>Tokens encrypted per user; no cross-user leak</t>
-        </is>
-      </c>
-      <c r="R70" s="3" t="inlineStr"/>
+          <t>Design reuses content-core + graphs/source.py</t>
+        </is>
+      </c>
+      <c r="R70" s="3" t="inlineStr">
+        <is>
+          <t>Blocked until WP2 users/tokens exist</t>
+        </is>
+      </c>
       <c r="S70" s="3" t="inlineStr"/>
     </row>
     <row r="71" ht="75" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -6441,18 +6568,18 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Frontend: Add from SharePoint / Link flow</t>
+          <t>SourceConnector interface + bulk job fan-out</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Purpose: ship the operator UX for connect → folder pick → select → progress, then chat across the pulled set.
-Steps: add sources steps UI; show per-doc progress; ensure i18n for all locales; group pulled docs for chat/search.</t>
+          <t>Purpose: one “add location” action becomes N document jobs with per-doc progress and partial failure tolerance.
+Steps: define authenticate/list_documents/fetch_document; extend source_commands for fan-out; ensure one bad file does not abort the batch.</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Sources UI flow</t>
+          <t>Connector API + bulk command</t>
         </is>
       </c>
       <c r="F71" s="22" t="inlineStr">
@@ -6460,14 +6587,14 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G71" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G71" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>7.2,7.3</t>
+          <t>7.0</t>
         </is>
       </c>
       <c r="I71" s="17" t="n">
@@ -6482,32 +6609,28 @@
       </c>
       <c r="M71" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N71" s="19" t="n">
-        <v>46276</v>
+        <v>46266</v>
       </c>
       <c r="O71" s="19" t="n">
-        <v>46281</v>
+        <v>46269</v>
       </c>
       <c r="P71" s="3" t="n"/>
       <c r="Q71" s="3" t="inlineStr">
         <is>
-          <t>User can chat across the whole pulled set</t>
-        </is>
-      </c>
-      <c r="R71" s="3" t="inlineStr">
-        <is>
-          <t>i18n required for all locales</t>
-        </is>
-      </c>
+          <t>Single failure does not abort batch; progress per document</t>
+        </is>
+      </c>
+      <c r="R71" s="3" t="inlineStr"/>
       <c r="S71" s="3" t="inlineStr"/>
     </row>
     <row r="72" ht="75" customHeight="1">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>7.6</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -6517,18 +6640,18 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>docs/CONNECTORS.md + WP5 review</t>
+          <t>SharePoint connector (Microsoft Graph)</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Purpose: document Entra scopes/consent and how to add a connector; close WP5 on acceptance criteria.
-Steps: write CONNECTORS.md; verify ACs; PR; human review stop.</t>
+          <t>Purpose: let an Entra-signed-in user pull an entire SharePoint folder into chat-able sources.
+Steps: OAuth on behalf of the user; least-privilege Sites/Files read scopes; enumerate folder; download supported files into existing ingestion; document admin consent.</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>docs/CONNECTORS.md; merged WP5</t>
+          <t>SharePointConnector</t>
         </is>
       </c>
       <c r="F72" s="22" t="inlineStr">
@@ -6536,21 +6659,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G72" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G72" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>7.4,7.5</t>
+          <t>7.1,4.7</t>
         </is>
       </c>
       <c r="I72" s="17" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="J72" s="17" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K72" s="17" t="n"/>
       <c r="L72" s="18" t="n">
@@ -6558,19 +6681,19 @@
       </c>
       <c r="M72" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N72" s="19" t="n">
-        <v>46281</v>
+        <v>46269</v>
       </c>
       <c r="O72" s="19" t="n">
-        <v>46282</v>
+        <v>46275</v>
       </c>
       <c r="P72" s="3" t="n"/>
       <c r="Q72" s="3" t="inlineStr">
         <is>
-          <t>All WP5 acceptance criteria pass</t>
+          <t>User connects SharePoint, picks folder, pulls all supported docs</t>
         </is>
       </c>
       <c r="R72" s="3" t="inlineStr"/>
@@ -6579,28 +6702,28 @@
     <row r="73" ht="75" customHeight="1">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>WP6 — Doc Processing Benchmarks</t>
+          <t>WP5 — External Source Connectors</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>WP6 kickoff + enumerate supported types</t>
+          <t>Generic DMS / multi-doc link connector</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Purpose: list what content-core actually supports today and what needs work (OCR, EPUB, upload HTML, etc.).
-Steps: inventory from real code/config; note gaps; create wp-6-benchmarks. Can run after WP0; needs target hardware for later measurement tasks.</t>
+          <t>Purpose: support folder URLs / IDs that resolve to many documents, with an extension point for other DMS systems.
+Steps: implement base multi-doc connector; keep the SourceConnector interface as the only required surface for new connectors.</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Type inventory</t>
+          <t>Generic multi-doc connector</t>
         </is>
       </c>
       <c r="F73" s="22" t="inlineStr">
@@ -6608,21 +6731,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G73" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G73" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="I73" s="17" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="J73" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K73" s="17" t="n"/>
       <c r="L73" s="18" t="n">
@@ -6630,53 +6753,49 @@
       </c>
       <c r="M73" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N73" s="19" t="n">
-        <v>46266</v>
+        <v>46273</v>
       </c>
       <c r="O73" s="19" t="n">
-        <v>46267</v>
+        <v>46275</v>
       </c>
       <c r="P73" s="3" t="n"/>
       <c r="Q73" s="3" t="inlineStr">
         <is>
-          <t>Supported types documented from real code</t>
-        </is>
-      </c>
-      <c r="R73" s="3" t="inlineStr">
-        <is>
-          <t>No guessed client-facing numbers</t>
-        </is>
-      </c>
+          <t>New connector = implement interface only</t>
+        </is>
+      </c>
+      <c r="R73" s="3" t="inlineStr"/>
       <c r="S73" s="3" t="inlineStr"/>
     </row>
     <row r="74" ht="75" customHeight="1">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.4</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>WP6 — Doc Processing Benchmarks</t>
+          <t>WP5 — External Source Connectors</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Build /benchmarks/ harness</t>
+          <t>Encrypted per-user token storage</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Purpose: produce repeatable measured metrics — not estimates — for ingestion, extraction, embedding, memory, and search/chat latency.
-Steps: build parameterized harness under /benchmarks/; output machine-readable reports.</t>
+          <t>Purpose: store connector OAuth tokens encrypted per user using existing encryption-key infrastructure.
+Steps: persist tokens encrypted; never share across users; respect source-system permissions (never fetch what the user cannot access).</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>/benchmarks/ harness</t>
+          <t>Encrypted token store</t>
         </is>
       </c>
       <c r="F74" s="22" t="inlineStr">
@@ -6684,21 +6803,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G74" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G74" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>7.2,2.8</t>
         </is>
       </c>
       <c r="I74" s="17" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="J74" s="17" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="K74" s="17" t="n"/>
       <c r="L74" s="18" t="n">
@@ -6706,19 +6825,19 @@
       </c>
       <c r="M74" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N74" s="19" t="n">
-        <v>46267</v>
+        <v>46275</v>
       </c>
       <c r="O74" s="19" t="n">
-        <v>46270</v>
+        <v>46276</v>
       </c>
       <c r="P74" s="3" t="n"/>
       <c r="Q74" s="3" t="inlineStr">
         <is>
-          <t>Harness runs repeatably and outputs a metrics report</t>
+          <t>Tokens encrypted per user; no cross-user leak</t>
         </is>
       </c>
       <c r="R74" s="3" t="inlineStr"/>
@@ -6727,28 +6846,28 @@
     <row r="75" ht="75" customHeight="1">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>WP6 — Doc Processing Benchmarks</t>
+          <t>WP5 — External Source Connectors</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Assemble representative corpus</t>
+          <t>Frontend: Add from SharePoint / Link flow</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Purpose: find empirical slowdown/failure points across sizes and types.
-Steps: assemble small/medium/large/very-large docs plus scanned PDF, audio, and web page; ensure corpus licensing is clean for redistribution in-repo if needed.</t>
+          <t>Purpose: ship the operator UX for connect → folder pick → select → progress, then chat across the pulled set.
+Steps: add sources steps UI; show per-doc progress; ensure i18n for all locales; group pulled docs for chat/search.</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Fixed corpus under benchmarks/</t>
+          <t>Sources UI flow</t>
         </is>
       </c>
       <c r="F75" s="22" t="inlineStr">
@@ -6763,14 +6882,14 @@
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.2,7.3</t>
         </is>
       </c>
       <c r="I75" s="17" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="J75" s="17" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="K75" s="17" t="n"/>
       <c r="L75" s="18" t="n">
@@ -6778,49 +6897,53 @@
       </c>
       <c r="M75" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N75" s="19" t="n">
-        <v>46270</v>
+        <v>46276</v>
       </c>
       <c r="O75" s="19" t="n">
-        <v>46273</v>
+        <v>46281</v>
       </c>
       <c r="P75" s="3" t="n"/>
       <c r="Q75" s="3" t="inlineStr">
         <is>
-          <t>Corpus covers the size/type matrix</t>
-        </is>
-      </c>
-      <c r="R75" s="3" t="inlineStr"/>
+          <t>User can chat across the whole pulled set</t>
+        </is>
+      </c>
+      <c r="R75" s="3" t="inlineStr">
+        <is>
+          <t>i18n required for all locales</t>
+        </is>
+      </c>
       <c r="S75" s="3" t="inlineStr"/>
     </row>
     <row r="76" ht="75" customHeight="1">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>7.6</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>WP6 — Doc Processing Benchmarks</t>
+          <t>WP5 — External Source Connectors</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Define accuracy methodology</t>
+          <t>docs/CONNECTORS.md + WP5 review</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Purpose: define how accuracy is measured so client claims are defensible.
-Steps: specify extraction fidelity, retrieval relevance (labeled Q&amp;A), and chat groundedness methods; report per model tier.</t>
+          <t>Purpose: document Entra scopes/consent and how to add a connector; close WP5 on acceptance criteria.
+Steps: write CONNECTORS.md; verify ACs; PR; human review stop.</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>Accuracy method doc section</t>
+          <t>docs/CONNECTORS.md; merged WP5</t>
         </is>
       </c>
       <c r="F76" s="22" t="inlineStr">
@@ -6835,7 +6958,7 @@
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.4,7.5</t>
         </is>
       </c>
       <c r="I76" s="17" t="n">
@@ -6854,15 +6977,15 @@
         </is>
       </c>
       <c r="N76" s="19" t="n">
-        <v>46270</v>
+        <v>46281</v>
       </c>
       <c r="O76" s="19" t="n">
-        <v>46273</v>
+        <v>46282</v>
       </c>
       <c r="P76" s="3" t="n"/>
       <c r="Q76" s="3" t="inlineStr">
         <is>
-          <t>Accuracy reported as method + numbers</t>
+          <t>All WP5 acceptance criteria pass</t>
         </is>
       </c>
       <c r="R76" s="3" t="inlineStr"/>
@@ -6871,7 +6994,7 @@
     <row r="77" ht="75" customHeight="1">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -6881,18 +7004,18 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Run ≥2 hardware profiles</t>
+          <t>WP6 kickoff + enumerate supported types</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Purpose: gather real numbers on bare-minimum and recommended hardware.
-Steps: run harness on both profiles; record figures; note local-model vs API-provider resource differences. Requires access to target hardware.</t>
+          <t>Purpose: list what content-core actually supports today and what needs work (OCR, EPUB, upload HTML, etc.).
+Steps: inventory from real code/config; note gaps; create wp-6-benchmarks. Can run after WP0; needs target hardware for later measurement tasks.</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Raw results JSON/CSV</t>
+          <t>Type inventory</t>
         </is>
       </c>
       <c r="F77" s="22" t="inlineStr">
@@ -6900,21 +7023,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G77" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G77" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>8.2,8.3</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="I77" s="17" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="J77" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K77" s="17" t="n"/>
       <c r="L77" s="18" t="n">
@@ -6926,20 +7049,20 @@
         </is>
       </c>
       <c r="N77" s="19" t="n">
-        <v>46273</v>
+        <v>46266</v>
       </c>
       <c r="O77" s="19" t="n">
-        <v>46276</v>
+        <v>46267</v>
       </c>
       <c r="P77" s="3" t="n"/>
       <c r="Q77" s="3" t="inlineStr">
         <is>
-          <t>Real measured numbers for both profiles</t>
+          <t>Supported types documented from real code</t>
         </is>
       </c>
       <c r="R77" s="3" t="inlineStr">
         <is>
-          <t>Hardware access is a dependency</t>
+          <t>No guessed client-facing numbers</t>
         </is>
       </c>
       <c r="S77" s="3" t="inlineStr"/>
@@ -6947,7 +7070,7 @@
     <row r="78" ht="75" customHeight="1">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -6957,18 +7080,18 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>docs/PERFORMANCE_AND_SIZING.md + review</t>
+          <t>Build /benchmarks/ harness</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Purpose: publish client-facing sizing guidance backed only by harness output.
-Steps: write types, limits, times, accuracy, min vs recommended hardware; peer review; merge.</t>
+          <t>Purpose: produce repeatable measured metrics — not estimates — for ingestion, extraction, embedding, memory, and search/chat latency.
+Steps: build parameterized harness under /benchmarks/; output machine-readable reports.</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>docs/PERFORMANCE_AND_SIZING.md</t>
+          <t>/benchmarks/ harness</t>
         </is>
       </c>
       <c r="F78" s="22" t="inlineStr">
@@ -6983,14 +7106,14 @@
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="I78" s="17" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="J78" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K78" s="17" t="n"/>
       <c r="L78" s="18" t="n">
@@ -7002,15 +7125,15 @@
         </is>
       </c>
       <c r="N78" s="19" t="n">
-        <v>46276</v>
+        <v>46267</v>
       </c>
       <c r="O78" s="19" t="n">
-        <v>46277</v>
+        <v>46270</v>
       </c>
       <c r="P78" s="3" t="n"/>
       <c r="Q78" s="3" t="inlineStr">
         <is>
-          <t>Doc contains measured numbers only</t>
+          <t>Harness runs repeatably and outputs a metrics report</t>
         </is>
       </c>
       <c r="R78" s="3" t="inlineStr"/>
@@ -7019,28 +7142,28 @@
     <row r="79" ht="75" customHeight="1">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>WP7 — Cross-platform Packaging</t>
+          <t>WP6 — Doc Processing Benchmarks</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>WP7 kickoff</t>
+          <t>Assemble representative corpus</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Purpose: package the real authenticated + branded app, not the pre-WP2 password prototype.
-Steps: create wp-7-packaging only after WP2 and WP3 are on main.</t>
+          <t>Purpose: find empirical slowdown/failure points across sizes and types.
+Steps: assemble small/medium/large/very-large docs plus scanned PDF, audio, and web page; ensure corpus licensing is clean for redistribution in-repo if needed.</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>Fixed corpus under benchmarks/</t>
         </is>
       </c>
       <c r="F79" s="22" t="inlineStr">
@@ -7055,14 +7178,14 @@
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>5.6,4.10</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="I79" s="17" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="J79" s="17" t="n">
-        <v>0.25</v>
+        <v>1.5</v>
       </c>
       <c r="K79" s="17" t="n"/>
       <c r="L79" s="18" t="n">
@@ -7074,15 +7197,15 @@
         </is>
       </c>
       <c r="N79" s="19" t="n">
-        <v>46283</v>
+        <v>46270</v>
       </c>
       <c r="O79" s="19" t="n">
-        <v>46283</v>
+        <v>46273</v>
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="inlineStr">
         <is>
-          <t>Starts only after branded + authenticated app exists</t>
+          <t>Corpus covers the size/type matrix</t>
         </is>
       </c>
       <c r="R79" s="3" t="inlineStr"/>
@@ -7091,28 +7214,28 @@
     <row r="80" ht="75" customHeight="1">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>WP7 — Cross-platform Packaging</t>
+          <t>WP6 — Doc Processing Benchmarks</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Verify Docker Compose on Windows + Linux</t>
+          <t>Define accuracy methodology</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Purpose: make containers the recommended identical path on both OSes.
-Steps: verify docker-compose and Dockerfile.single on Docker Desktop/WSL2 and Linux; document as primary deploy path.</t>
+          <t>Purpose: define how accuracy is measured so client claims are defensible.
+Steps: specify extraction fidelity, retrieval relevance (labeled Q&amp;A), and chat groundedness methods; report per model tier.</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>Verified container deploy</t>
+          <t>Accuracy method doc section</t>
         </is>
       </c>
       <c r="F80" s="22" t="inlineStr">
@@ -7120,21 +7243,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G80" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G80" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="I80" s="17" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="J80" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K80" s="17" t="n"/>
       <c r="L80" s="18" t="n">
@@ -7142,19 +7265,19 @@
       </c>
       <c r="M80" s="3" t="inlineStr">
         <is>
-          <t>DevOps / Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N80" s="19" t="n">
-        <v>46283</v>
+        <v>46270</v>
       </c>
       <c r="O80" s="19" t="n">
-        <v>46287</v>
+        <v>46273</v>
       </c>
       <c r="P80" s="3" t="n"/>
       <c r="Q80" s="3" t="inlineStr">
         <is>
-          <t>Container deployment verified on both OSes</t>
+          <t>Accuracy reported as method + numbers</t>
         </is>
       </c>
       <c r="R80" s="3" t="inlineStr"/>
@@ -7163,28 +7286,28 @@
     <row r="81" ht="75" customHeight="1">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>WP7 — Cross-platform Packaging</t>
+          <t>WP6 — Doc Processing Benchmarks</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Native Linux install path (systemd)</t>
+          <t>Run ≥2 hardware profiles</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Purpose: support customers who refuse containers.
-Steps: systemd units + install script; document dependencies for common distros; verify on at least one distro.</t>
+          <t>Purpose: gather real numbers on bare-minimum and recommended hardware.
+Steps: run harness on both profiles; record figures; note local-model vs API-provider resource differences. Requires access to target hardware.</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Linux native docs + scripts</t>
+          <t>Raw results JSON/CSV</t>
         </is>
       </c>
       <c r="F81" s="22" t="inlineStr">
@@ -7192,21 +7315,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G81" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G81" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.2,8.3</t>
         </is>
       </c>
       <c r="I81" s="17" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="J81" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K81" s="17" t="n"/>
       <c r="L81" s="18" t="n">
@@ -7214,49 +7337,53 @@
       </c>
       <c r="M81" s="3" t="inlineStr">
         <is>
-          <t>DevOps / Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N81" s="19" t="n">
-        <v>46287</v>
+        <v>46273</v>
       </c>
       <c r="O81" s="19" t="n">
-        <v>46289</v>
+        <v>46276</v>
       </c>
       <c r="P81" s="3" t="n"/>
       <c r="Q81" s="3" t="inlineStr">
         <is>
-          <t>Verified on ≥1 Linux distro</t>
-        </is>
-      </c>
-      <c r="R81" s="3" t="inlineStr"/>
+          <t>Real measured numbers for both profiles</t>
+        </is>
+      </c>
+      <c r="R81" s="3" t="inlineStr">
+        <is>
+          <t>Hardware access is a dependency</t>
+        </is>
+      </c>
       <c r="S81" s="3" t="inlineStr"/>
     </row>
     <row r="82" ht="75" customHeight="1">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>9.3</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>WP7 — Cross-platform Packaging</t>
+          <t>WP6 — Doc Processing Benchmarks</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Native Windows Service path</t>
+          <t>docs/PERFORMANCE_AND_SIZING.md + review</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Purpose: support Windows Server native installs.
-Steps: Windows Service wrapper; SurrealDB-on-Windows notes; frontend serve docs; verify on Windows Server or equivalent.</t>
+          <t>Purpose: publish client-facing sizing guidance backed only by harness output.
+Steps: write types, limits, times, accuracy, min vs recommended hardware; peer review; merge.</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>Windows native docs + scripts</t>
+          <t>docs/PERFORMANCE_AND_SIZING.md</t>
         </is>
       </c>
       <c r="F82" s="22" t="inlineStr">
@@ -7264,21 +7391,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G82" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G82" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="I82" s="17" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="J82" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K82" s="17" t="n"/>
       <c r="L82" s="18" t="n">
@@ -7286,19 +7413,19 @@
       </c>
       <c r="M82" s="3" t="inlineStr">
         <is>
-          <t>DevOps / Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N82" s="19" t="n">
-        <v>46287</v>
+        <v>46276</v>
       </c>
       <c r="O82" s="19" t="n">
-        <v>46289</v>
+        <v>46277</v>
       </c>
       <c r="P82" s="3" t="n"/>
       <c r="Q82" s="3" t="inlineStr">
         <is>
-          <t>Verified on Windows Server or equivalent</t>
+          <t>Doc contains measured numbers only</t>
         </is>
       </c>
       <c r="R82" s="3" t="inlineStr"/>
@@ -7307,7 +7434,7 @@
     <row r="83" ht="75" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -7317,18 +7444,18 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Installer helper CLI (interactive + non-interactive)</t>
+          <t>WP7 kickoff</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Purpose: let a non-expert stand up a branded client instance without hand-editing half a dozen files.
-Steps: CLI for prereq check → collect brand/Entra/provider/DB/encryption → write config → migrate → start → health check; add scripted/non-interactive mode for repeatable installs.</t>
+          <t>Purpose: package the real authenticated + branded app, not the pre-WP2 password prototype.
+Steps: create wp-7-packaging only after WP2 and WP3 are on main.</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>onboard/install CLI</t>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F83" s="22" t="inlineStr">
@@ -7336,21 +7463,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G83" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G83" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>9.1,5.4</t>
+          <t>5.6,4.10</t>
         </is>
       </c>
       <c r="I83" s="17" t="n">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="J83" s="17" t="n">
-        <v>4</v>
+        <v>0.25</v>
       </c>
       <c r="K83" s="17" t="n"/>
       <c r="L83" s="18" t="n">
@@ -7358,32 +7485,28 @@
       </c>
       <c r="M83" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N83" s="19" t="n">
-        <v>46289</v>
+        <v>46283</v>
       </c>
       <c r="O83" s="19" t="n">
-        <v>46295</v>
+        <v>46283</v>
       </c>
       <c r="P83" s="3" t="n"/>
       <c r="Q83" s="3" t="inlineStr">
         <is>
-          <t>Full install in both modes; scripted branded client stand-up works</t>
-        </is>
-      </c>
-      <c r="R83" s="3" t="inlineStr">
-        <is>
-          <t>Deployment counterpart to WP3 theming</t>
-        </is>
-      </c>
+          <t>Starts only after branded + authenticated app exists</t>
+        </is>
+      </c>
+      <c r="R83" s="3" t="inlineStr"/>
       <c r="S83" s="3" t="inlineStr"/>
     </row>
     <row r="84" ht="75" customHeight="1">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -7393,18 +7516,18 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>docs/DEPLOYMENT.md + WP7 review</t>
+          <t>Verify Docker Compose on Windows + Linux</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Purpose: one operator guide for container + native + CLI paths.
-Steps: write DEPLOYMENT.md; verify WP7 ACs; PR; human review.</t>
+          <t>Purpose: make containers the recommended identical path on both OSes.
+Steps: verify docker-compose and Dockerfile.single on Docker Desktop/WSL2 and Linux; document as primary deploy path.</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>docs/DEPLOYMENT.md</t>
+          <t>Verified container deploy</t>
         </is>
       </c>
       <c r="F84" s="22" t="inlineStr">
@@ -7412,21 +7535,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G84" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G84" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>9.2,9.3,9.4</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="I84" s="17" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="J84" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K84" s="17" t="n"/>
       <c r="L84" s="18" t="n">
@@ -7434,19 +7557,19 @@
       </c>
       <c r="M84" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>DevOps / Engineer</t>
         </is>
       </c>
       <c r="N84" s="19" t="n">
-        <v>46295</v>
+        <v>46283</v>
       </c>
       <c r="O84" s="19" t="n">
-        <v>46296</v>
+        <v>46287</v>
       </c>
       <c r="P84" s="3" t="n"/>
       <c r="Q84" s="3" t="inlineStr">
         <is>
-          <t>All WP7 acceptance criteria pass</t>
+          <t>Container deployment verified on both OSes</t>
         </is>
       </c>
       <c r="R84" s="3" t="inlineStr"/>
@@ -7455,28 +7578,28 @@
     <row r="85" ht="75" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>WP8 — Onboarding &amp; In-app Help</t>
+          <t>WP7 — Cross-platform Packaging</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>WP8 kickoff (LAST)</t>
+          <t>Native Linux install path (systemd)</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Purpose: build onboarding against final flows only — wizard/tour copy must match the shipped product.
-Steps: create wp-8-onboarding after WP2/3/5/7 are stable on main.</t>
+          <t>Purpose: support customers who refuse containers.
+Steps: systemd units + install script; document dependencies for common distros; verify on at least one distro.</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>Linux native docs + scripts</t>
         </is>
       </c>
       <c r="F85" s="22" t="inlineStr">
@@ -7491,14 +7614,14 @@
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>9.5,7.6,5.6</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="I85" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="J85" s="17" t="n">
         <v>2</v>
-      </c>
-      <c r="J85" s="17" t="n">
-        <v>0.25</v>
       </c>
       <c r="K85" s="17" t="n"/>
       <c r="L85" s="18" t="n">
@@ -7506,53 +7629,49 @@
       </c>
       <c r="M85" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>DevOps / Engineer</t>
         </is>
       </c>
       <c r="N85" s="19" t="n">
-        <v>46297</v>
+        <v>46287</v>
       </c>
       <c r="O85" s="19" t="n">
-        <v>46297</v>
+        <v>46289</v>
       </c>
       <c r="P85" s="3" t="n"/>
       <c r="Q85" s="3" t="inlineStr">
         <is>
-          <t>Built against final UX</t>
-        </is>
-      </c>
-      <c r="R85" s="3" t="inlineStr">
-        <is>
-          <t>Must be last in the program sequence</t>
-        </is>
-      </c>
+          <t>Verified on ≥1 Linux distro</t>
+        </is>
+      </c>
+      <c r="R85" s="3" t="inlineStr"/>
       <c r="S85" s="3" t="inlineStr"/>
     </row>
     <row r="86" ht="75" customHeight="1">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>WP8 — Onboarding &amp; In-app Help</t>
+          <t>WP7 — Cross-platform Packaging</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>First-run / admin setup wizard</t>
+          <t>Native Windows Service path</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Purpose: take a fresh instance to a working configured app without tribal knowledge.
-Steps: detect fresh instance; guide providers/keys, models, brand (admin), connect a source, create first notebook; all copy via i18n.</t>
+          <t>Purpose: support Windows Server native installs.
+Steps: Windows Service wrapper; SurrealDB-on-Windows notes; frontend serve docs; verify on Windows Server or equivalent.</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>Setup wizard</t>
+          <t>Windows native docs + scripts</t>
         </is>
       </c>
       <c r="F86" s="22" t="inlineStr">
@@ -7560,21 +7679,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G86" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G86" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="I86" s="17" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="J86" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K86" s="17" t="n"/>
       <c r="L86" s="18" t="n">
@@ -7582,19 +7701,19 @@
       </c>
       <c r="M86" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>DevOps / Engineer</t>
         </is>
       </c>
       <c r="N86" s="19" t="n">
-        <v>46297</v>
+        <v>46287</v>
       </c>
       <c r="O86" s="19" t="n">
-        <v>46302</v>
+        <v>46289</v>
       </c>
       <c r="P86" s="3" t="n"/>
       <c r="Q86" s="3" t="inlineStr">
         <is>
-          <t>Completing the wizard leaves a working configured app</t>
+          <t>Verified on Windows Server or equivalent</t>
         </is>
       </c>
       <c r="R86" s="3" t="inlineStr"/>
@@ -7603,28 +7722,28 @@
     <row r="87" ht="75" customHeight="1">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>9.4</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>WP8 — Onboarding &amp; In-app Help</t>
+          <t>WP7 — Cross-platform Packaging</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>User guided tour (core loop)</t>
+          <t>Installer helper CLI (interactive + non-interactive)</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Purpose: teach the core loop — add source → search → chat → transform → podcast — with an accessible spotlight tour.
-Steps: implement dismissible/resumable tour; keep steps short; i18n all locales.</t>
+          <t>Purpose: let a non-expert stand up a branded client instance without hand-editing half a dozen files.
+Steps: CLI for prereq check → collect brand/Entra/provider/DB/encryption → write config → migrate → start → health check; add scripted/non-interactive mode for repeatable installs.</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Guided tour</t>
+          <t>onboard/install CLI</t>
         </is>
       </c>
       <c r="F87" s="22" t="inlineStr">
@@ -7632,21 +7751,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G87" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G87" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>9.1,5.4</t>
         </is>
       </c>
       <c r="I87" s="17" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="J87" s="17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K87" s="17" t="n"/>
       <c r="L87" s="18" t="n">
@@ -7654,49 +7773,53 @@
       </c>
       <c r="M87" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N87" s="19" t="n">
-        <v>46302</v>
+        <v>46289</v>
       </c>
       <c r="O87" s="19" t="n">
-        <v>46304</v>
+        <v>46295</v>
       </c>
       <c r="P87" s="3" t="n"/>
       <c r="Q87" s="3" t="inlineStr">
         <is>
-          <t>New user can complete the core-loop tour</t>
-        </is>
-      </c>
-      <c r="R87" s="3" t="inlineStr"/>
+          <t>Full install in both modes; scripted branded client stand-up works</t>
+        </is>
+      </c>
+      <c r="R87" s="3" t="inlineStr">
+        <is>
+          <t>Deployment counterpart to WP3 theming</t>
+        </is>
+      </c>
       <c r="S87" s="3" t="inlineStr"/>
     </row>
     <row r="88" ht="75" customHeight="1">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>WP8 — Onboarding &amp; In-app Help</t>
+          <t>WP7 — Cross-platform Packaging</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>Contextual tooltips + empty states + help surface</t>
+          <t>docs/DEPLOYMENT.md + WP7 review</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Purpose: remove dead-ends for new users on every main screen.
-Steps: tooltips on non-obvious controls; useful empty states; persistent help (docs, shortcuts, restart tour, BrandConfig support URL); all strings in i18n.</t>
+          <t>Purpose: one operator guide for container + native + CLI paths.
+Steps: write DEPLOYMENT.md; verify WP7 ACs; PR; human review.</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>Tooltips/empty states/help</t>
+          <t>docs/DEPLOYMENT.md</t>
         </is>
       </c>
       <c r="F88" s="22" t="inlineStr">
@@ -7704,21 +7827,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G88" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G88" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>9.2,9.3,9.4</t>
         </is>
       </c>
       <c r="I88" s="17" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="J88" s="17" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="K88" s="17" t="n"/>
       <c r="L88" s="18" t="n">
@@ -7726,32 +7849,28 @@
       </c>
       <c r="M88" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N88" s="19" t="n">
-        <v>46304</v>
+        <v>46295</v>
       </c>
       <c r="O88" s="19" t="n">
-        <v>46309</v>
+        <v>46296</v>
       </c>
       <c r="P88" s="3" t="n"/>
       <c r="Q88" s="3" t="inlineStr">
         <is>
-          <t>All copy in i18n; help reachable everywhere</t>
-        </is>
-      </c>
-      <c r="R88" s="3" t="inlineStr">
-        <is>
-          <t>Locale parity required across all locales</t>
-        </is>
-      </c>
+          <t>All WP7 acceptance criteria pass</t>
+        </is>
+      </c>
+      <c r="R88" s="3" t="inlineStr"/>
       <c r="S88" s="3" t="inlineStr"/>
     </row>
     <row r="89" ht="75" customHeight="1">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -7761,18 +7880,18 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>docs/ONBOARDING.md + program close review</t>
+          <t>WP8 kickoff (LAST)</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Purpose: document onboarding structure and verify program-level definition of done.
-Steps: write ONBOARDING.md; confirm a new client can be stood up by config + installer only (branded, Entra-auth’d, connectors, Windows/Linux) without per-client code rebuilds.</t>
+          <t>Purpose: build onboarding against final flows only — wizard/tour copy must match the shipped product.
+Steps: create wp-8-onboarding after WP2/3/5/7 are stable on main.</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>docs/ONBOARDING.md; program DoD check</t>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F89" s="22" t="inlineStr">
@@ -7787,14 +7906,14 @@
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>9.5,7.6,5.6</t>
         </is>
       </c>
       <c r="I89" s="17" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J89" s="17" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="K89" s="17" t="n"/>
       <c r="L89" s="18" t="n">
@@ -7802,26 +7921,322 @@
       </c>
       <c r="M89" s="3" t="inlineStr">
         <is>
-          <t>Engineering Lead</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N89" s="19" t="n">
-        <v>46309</v>
+        <v>46297</v>
       </c>
       <c r="O89" s="19" t="n">
-        <v>46310</v>
+        <v>46297</v>
       </c>
       <c r="P89" s="3" t="n"/>
       <c r="Q89" s="3" t="inlineStr">
         <is>
+          <t>Built against final UX</t>
+        </is>
+      </c>
+      <c r="R89" s="3" t="inlineStr">
+        <is>
+          <t>Must be last in the program sequence</t>
+        </is>
+      </c>
+      <c r="S89" s="3" t="inlineStr"/>
+    </row>
+    <row r="90" ht="75" customHeight="1">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>WP8 — Onboarding &amp; In-app Help</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>First-run / admin setup wizard</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: take a fresh instance to a working configured app without tribal knowledge.
+Steps: detect fresh instance; guide providers/keys, models, brand (admin), connect a source, create first notebook; all copy via i18n.</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>Setup wizard</t>
+        </is>
+      </c>
+      <c r="F90" s="22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G90" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H90" s="3" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="I90" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="J90" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K90" s="17" t="n"/>
+      <c r="L90" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M90" s="3" t="inlineStr">
+        <is>
+          <t>Frontend Engineer</t>
+        </is>
+      </c>
+      <c r="N90" s="19" t="n">
+        <v>46297</v>
+      </c>
+      <c r="O90" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="P90" s="3" t="n"/>
+      <c r="Q90" s="3" t="inlineStr">
+        <is>
+          <t>Completing the wizard leaves a working configured app</t>
+        </is>
+      </c>
+      <c r="R90" s="3" t="inlineStr"/>
+      <c r="S90" s="3" t="inlineStr"/>
+    </row>
+    <row r="91" ht="75" customHeight="1">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>WP8 — Onboarding &amp; In-app Help</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>User guided tour (core loop)</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: teach the core loop — add source → search → chat → transform → podcast — with an accessible spotlight tour.
+Steps: implement dismissible/resumable tour; keep steps short; i18n all locales.</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>Guided tour</t>
+        </is>
+      </c>
+      <c r="F91" s="22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G91" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H91" s="3" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="I91" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="J91" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K91" s="17" t="n"/>
+      <c r="L91" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" s="3" t="inlineStr">
+        <is>
+          <t>Frontend Engineer</t>
+        </is>
+      </c>
+      <c r="N91" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="O91" s="19" t="n">
+        <v>46304</v>
+      </c>
+      <c r="P91" s="3" t="n"/>
+      <c r="Q91" s="3" t="inlineStr">
+        <is>
+          <t>New user can complete the core-loop tour</t>
+        </is>
+      </c>
+      <c r="R91" s="3" t="inlineStr"/>
+      <c r="S91" s="3" t="inlineStr"/>
+    </row>
+    <row r="92" ht="75" customHeight="1">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>WP8 — Onboarding &amp; In-app Help</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>Contextual tooltips + empty states + help surface</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: remove dead-ends for new users on every main screen.
+Steps: tooltips on non-obvious controls; useful empty states; persistent help (docs, shortcuts, restart tour, BrandConfig support URL); all strings in i18n.</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>Tooltips/empty states/help</t>
+        </is>
+      </c>
+      <c r="F92" s="22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G92" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H92" s="3" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="I92" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="J92" s="17" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K92" s="17" t="n"/>
+      <c r="L92" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M92" s="3" t="inlineStr">
+        <is>
+          <t>Frontend Engineer</t>
+        </is>
+      </c>
+      <c r="N92" s="19" t="n">
+        <v>46304</v>
+      </c>
+      <c r="O92" s="19" t="n">
+        <v>46309</v>
+      </c>
+      <c r="P92" s="3" t="n"/>
+      <c r="Q92" s="3" t="inlineStr">
+        <is>
+          <t>All copy in i18n; help reachable everywhere</t>
+        </is>
+      </c>
+      <c r="R92" s="3" t="inlineStr">
+        <is>
+          <t>Locale parity required across all locales</t>
+        </is>
+      </c>
+      <c r="S92" s="3" t="inlineStr"/>
+    </row>
+    <row r="93" ht="75" customHeight="1">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>10.4</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>WP8 — Onboarding &amp; In-app Help</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>docs/ONBOARDING.md + program close review</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: document onboarding structure and verify program-level definition of done.
+Steps: write ONBOARDING.md; confirm a new client can be stood up by config + installer only (branded, Entra-auth’d, connectors, Windows/Linux) without per-client code rebuilds.</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>docs/ONBOARDING.md; program DoD check</t>
+        </is>
+      </c>
+      <c r="F93" s="22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G93" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H93" s="3" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="I93" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="J93" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K93" s="17" t="n"/>
+      <c r="L93" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M93" s="3" t="inlineStr">
+        <is>
+          <t>Engineering Lead</t>
+        </is>
+      </c>
+      <c r="N93" s="19" t="n">
+        <v>46309</v>
+      </c>
+      <c r="O93" s="19" t="n">
+        <v>46310</v>
+      </c>
+      <c r="P93" s="3" t="n"/>
+      <c r="Q93" s="3" t="inlineStr">
+        <is>
           <t>All WP8 ACs + program definition of done satisfied</t>
         </is>
       </c>
-      <c r="R89" s="3" t="inlineStr"/>
-      <c r="S89" s="3" t="inlineStr"/>
+      <c r="R93" s="3" t="inlineStr"/>
+      <c r="S93" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A5:S89"/>
+  <autoFilter ref="A5:S93"/>
   <mergeCells count="3">
     <mergeCell ref="A3:S3"/>
     <mergeCell ref="A2:S2"/>
@@ -7892,7 +8307,7 @@
           <t>Clean build reproducible from docs/DEV_SETUP.md</t>
         </is>
       </c>
-      <c r="C4" s="26" t="inlineStr">
+      <c r="C4" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7915,7 +8330,7 @@
           <t>upstream-base tag exists; upstream remote configured</t>
         </is>
       </c>
-      <c r="C5" s="26" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7942,7 +8357,7 @@
           <t>Characterization tests: ingestion, search, chat, notebook CRUD</t>
         </is>
       </c>
-      <c r="C6" s="26" t="inlineStr">
+      <c r="C6" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7965,7 +8380,7 @@
           <t>CI runs on PR and blocks merge on failure</t>
         </is>
       </c>
-      <c r="C7" s="26" t="inlineStr">
+      <c r="C7" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7988,7 +8403,7 @@
           <t>License scan runs in CI and passes</t>
         </is>
       </c>
-      <c r="C8" s="26" t="inlineStr">
+      <c r="C8" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8011,7 +8426,7 @@
           <t>LICENSE retains upstream copyright + our copyright</t>
         </is>
       </c>
-      <c r="C9" s="26" t="inlineStr">
+      <c r="C9" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8038,7 +8453,7 @@
           <t>THIRD-PARTY-NOTICES.md complete and reproducible</t>
         </is>
       </c>
-      <c r="C10" s="26" t="inlineStr">
+      <c r="C10" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8065,7 +8480,7 @@
           <t>SurrealDB BSL entry present and accurate</t>
         </is>
       </c>
-      <c r="C11" s="26" t="inlineStr">
+      <c r="C11" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8088,7 +8503,7 @@
           <t>pycountry unmodified; CI asserts</t>
         </is>
       </c>
-      <c r="C12" s="26" t="inlineStr">
+      <c r="C12" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8111,7 +8526,7 @@
           <t>docs/PROVIDER_TERMS.md exists</t>
         </is>
       </c>
-      <c r="C13" s="26" t="inlineStr">
+      <c r="C13" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8138,7 +8553,7 @@
           <t>No secrets committed; encryption key handling documented</t>
         </is>
       </c>
-      <c r="C14" s="26" t="inlineStr">
+      <c r="C14" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8161,7 +8576,7 @@
           <t>Tenancy model chosen and documented</t>
         </is>
       </c>
-      <c r="C15" s="26" t="inlineStr">
+      <c r="C15" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8188,7 +8603,7 @@
           <t>Login via real Entra account E2E</t>
         </is>
       </c>
-      <c r="C16" s="27" t="inlineStr">
+      <c r="C16" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8211,7 +8626,7 @@
           <t>Every API request validates Entra JWT (iss/aud/sig/exp)</t>
         </is>
       </c>
-      <c r="C17" s="27" t="inlineStr">
+      <c r="C17" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8230,7 +8645,7 @@
           <t>Users JIT-provisioned; user record after first login</t>
         </is>
       </c>
-      <c r="C18" s="27" t="inlineStr">
+      <c r="C18" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8249,7 +8664,7 @@
           <t>Roles enforced on sensitive routes (403)</t>
         </is>
       </c>
-      <c r="C19" s="27" t="inlineStr">
+      <c r="C19" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8268,7 +8683,7 @@
           <t>Users only see own notebooks/sources</t>
         </is>
       </c>
-      <c r="C20" s="27" t="inlineStr">
+      <c r="C20" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8287,7 +8702,7 @@
           <t>Password provider still works as local-dev fallback</t>
         </is>
       </c>
-      <c r="C21" s="27" t="inlineStr">
+      <c r="C21" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8306,7 +8721,7 @@
           <t>Second provider needs no route-handler changes (stub)</t>
         </is>
       </c>
-      <c r="C22" s="27" t="inlineStr">
+      <c r="C22" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8325,7 +8740,7 @@
           <t>docs/AUTH.md complete</t>
         </is>
       </c>
-      <c r="C23" s="27" t="inlineStr">
+      <c r="C23" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8344,7 +8759,7 @@
           <t>FRONTEND_MAP.md complete with where-to-change table</t>
         </is>
       </c>
-      <c r="C24" s="27" t="inlineStr">
+      <c r="C24" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8363,7 +8778,7 @@
           <t>New client branded by config only (two brands, same build)</t>
         </is>
       </c>
-      <c r="C25" s="27" t="inlineStr">
+      <c r="C25" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8382,7 +8797,7 @@
           <t>Hardcoded brand strings/assets read from BrandConfig</t>
         </is>
       </c>
-      <c r="C26" s="27" t="inlineStr">
+      <c r="C26" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8401,7 +8816,7 @@
           <t>Dark/light both themed correctly</t>
         </is>
       </c>
-      <c r="C27" s="27" t="inlineStr">
+      <c r="C27" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8420,7 +8835,7 @@
           <t>Every router/endpoint documented with auth + models</t>
         </is>
       </c>
-      <c r="C28" s="27" t="inlineStr">
+      <c r="C28" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8439,7 +8854,7 @@
           <t>Every domain model and graph documented</t>
         </is>
       </c>
-      <c r="C29" s="27" t="inlineStr">
+      <c r="C29" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8458,7 +8873,7 @@
           <t>Five how-to-add-X playbooks present</t>
         </is>
       </c>
-      <c r="C30" s="27" t="inlineStr">
+      <c r="C30" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8477,7 +8892,7 @@
           <t>New engineer can locate changes using only BACKEND_MAP</t>
         </is>
       </c>
-      <c r="C31" s="27" t="inlineStr">
+      <c r="C31" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8496,7 +8911,7 @@
           <t>SharePoint connect → folder → pull all supported docs</t>
         </is>
       </c>
-      <c r="C32" s="27" t="inlineStr">
+      <c r="C32" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8515,7 +8930,7 @@
           <t>Ingestion reuses existing pipeline</t>
         </is>
       </c>
-      <c r="C33" s="27" t="inlineStr">
+      <c r="C33" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8534,7 +8949,7 @@
           <t>Batch per-doc progress; single failure non-fatal</t>
         </is>
       </c>
-      <c r="C34" s="27" t="inlineStr">
+      <c r="C34" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8553,7 +8968,7 @@
           <t>Chat across whole pulled set</t>
         </is>
       </c>
-      <c r="C35" s="27" t="inlineStr">
+      <c r="C35" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8572,7 +8987,7 @@
           <t>Tokens encrypted per user; source permissions respected</t>
         </is>
       </c>
-      <c r="C36" s="27" t="inlineStr">
+      <c r="C36" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8591,7 +9006,7 @@
           <t>New connector = SourceConnector interface only</t>
         </is>
       </c>
-      <c r="C37" s="27" t="inlineStr">
+      <c r="C37" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8610,7 +9025,7 @@
           <t>docs/CONNECTORS.md complete</t>
         </is>
       </c>
-      <c r="C38" s="27" t="inlineStr">
+      <c r="C38" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8629,7 +9044,7 @@
           <t>Benchmark harness repeatable with metrics report</t>
         </is>
       </c>
-      <c r="C39" s="27" t="inlineStr">
+      <c r="C39" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8648,7 +9063,7 @@
           <t>PERFORMANCE_AND_SIZING.md has measured numbers (2 profiles)</t>
         </is>
       </c>
-      <c r="C40" s="27" t="inlineStr">
+      <c r="C40" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8667,7 +9082,7 @@
           <t>Supported types + tested size limits + failure points</t>
         </is>
       </c>
-      <c r="C41" s="27" t="inlineStr">
+      <c r="C41" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8686,7 +9101,7 @@
           <t>Accuracy methodology + results per model tier</t>
         </is>
       </c>
-      <c r="C42" s="27" t="inlineStr">
+      <c r="C42" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8705,7 +9120,7 @@
           <t>Min vs recommended hardware justified by numbers</t>
         </is>
       </c>
-      <c r="C43" s="27" t="inlineStr">
+      <c r="C43" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8724,7 +9139,7 @@
           <t>Container deploy verified Windows + Linux</t>
         </is>
       </c>
-      <c r="C44" s="27" t="inlineStr">
+      <c r="C44" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8743,7 +9158,7 @@
           <t>Native install documented/verified Linux + Windows</t>
         </is>
       </c>
-      <c r="C45" s="27" t="inlineStr">
+      <c r="C45" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8762,7 +9177,7 @@
           <t>Installer CLI full install interactive + non-interactive</t>
         </is>
       </c>
-      <c r="C46" s="27" t="inlineStr">
+      <c r="C46" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8781,7 +9196,7 @@
           <t>Scripted install stands up branded client E2E</t>
         </is>
       </c>
-      <c r="C47" s="27" t="inlineStr">
+      <c r="C47" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8800,7 +9215,7 @@
           <t>docs/DEPLOYMENT.md complete</t>
         </is>
       </c>
-      <c r="C48" s="27" t="inlineStr">
+      <c r="C48" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8819,7 +9234,7 @@
           <t>Fresh instance launches setup wizard → working app</t>
         </is>
       </c>
-      <c r="C49" s="27" t="inlineStr">
+      <c r="C49" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8838,7 +9253,7 @@
           <t>Guided tour of core loop completable</t>
         </is>
       </c>
-      <c r="C50" s="27" t="inlineStr">
+      <c r="C50" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8857,7 +9272,7 @@
           <t>Contextual tooltips; all copy in i18n</t>
         </is>
       </c>
-      <c r="C51" s="27" t="inlineStr">
+      <c r="C51" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8876,7 +9291,7 @@
           <t>Every main screen useful empty state</t>
         </is>
       </c>
-      <c r="C52" s="27" t="inlineStr">
+      <c r="C52" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8895,7 +9310,7 @@
           <t>Tour dismissible/resumable; help surface everywhere</t>
         </is>
       </c>
-      <c r="C53" s="27" t="inlineStr">
+      <c r="C53" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8914,7 +9329,7 @@
           <t>docs/ONBOARDING.md complete</t>
         </is>
       </c>
-      <c r="C54" s="27" t="inlineStr">
+      <c r="C54" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8933,7 +9348,7 @@
           <t>New client by config + installer only (no per-client rebuild)</t>
         </is>
       </c>
-      <c r="C55" s="27" t="inlineStr">
+      <c r="C55" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8956,7 +9371,7 @@
           <t>Licensing compliant and drift-guarded</t>
         </is>
       </c>
-      <c r="C56" s="26" t="inlineStr">
+      <c r="C56" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8979,7 +9394,7 @@
           <t>Real performance/sizing numbers for clients</t>
         </is>
       </c>
-      <c r="C57" s="27" t="inlineStr">
+      <c r="C57" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9002,7 +9417,7 @@
           <t>Backend + frontend fully mapped</t>
         </is>
       </c>
-      <c r="C58" s="27" t="inlineStr">
+      <c r="C58" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9043,12 +9458,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="27" t="inlineStr">
         <is>
           <t>Topic</t>
         </is>
       </c>
-      <c r="B3" s="28" t="inlineStr">
+      <c r="B3" s="27" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>

</xml_diff>

<commit_message>
docs(wp2b): track sharing follow-ons in WBS 4.20-4.22
Record Entra group sync, Graph directory picker, and public-link/reshare/ownership-transfer as Pending carry-forward tasks; mark WP2b 4.15-4.18 Done and regenerate the commercialization Excel workbook.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/commercialization/Open-Notebook-Commercialization-WBS-Task-Schedule.xlsx
+++ b/docs/commercialization/Open-Notebook-Commercialization-WBS-Task-Schedule.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimating Assumptions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'WBS Task List'!$A$5:$S$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'WBS Task List'!$A$5:$S$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -138,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -196,6 +196,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -570,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -834,47 +837,41 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>WP3 — Frontend Map + White-label</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Pending</t>
+          <t>WP2b — Sharing &amp; Groups</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>81</v>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>74</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>72</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>10.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>After WP2 (admin UI optional)</t>
-        </is>
-      </c>
+        <v>0.9837837837837837</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>WP4 — Backend/API Documentation</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Pending</t>
+          <t>Carry-forward / Sharing Follow-through</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Open follow-ups</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
@@ -882,21 +879,17 @@
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>6.2</v>
+        <v>7</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Can parallel after WP0; better after WP2</t>
-        </is>
-      </c>
+      <c r="G12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>WP5 — External Source Connectors</t>
+          <t>WP3 — Frontend Map + White-label</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -905,7 +898,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>120</v>
+        <v>81</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
@@ -913,21 +906,21 @@
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>15</v>
+        <v>10.2</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Hard-blocked on WP2 OAuth users</t>
+          <t>After WP2 (admin UI optional)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>WP6 — Doc Processing Benchmarks</t>
+          <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -936,7 +929,7 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>84</v>
+        <v>49</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
@@ -944,21 +937,21 @@
         </is>
       </c>
       <c r="E14" s="3" t="n">
-        <v>10.5</v>
+        <v>6.2</v>
       </c>
       <c r="F14" s="5" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Needs target hardware</t>
+          <t>Can parallel after WP0; better after WP2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>WP7 — Cross-platform Packaging</t>
+          <t>WP5 — External Source Connectors</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
@@ -967,7 +960,7 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
@@ -975,21 +968,21 @@
         </is>
       </c>
       <c r="E15" s="3" t="n">
-        <v>11.2</v>
+        <v>15</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>After WP2+WP3</t>
+          <t>Hard-blocked on WP2 OAuth users</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>WP8 — Onboarding &amp; In-app Help</t>
+          <t>WP6 — Doc Processing Benchmarks</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -998,7 +991,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
@@ -1006,84 +999,126 @@
         </is>
       </c>
       <c r="E16" s="3" t="n">
-        <v>8.800000000000001</v>
+        <v>10.5</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>0</v>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
+          <t>Needs target hardware</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>WP7 — Cross-platform Packaging</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>After WP2+WP3</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>WP8 — Onboarding &amp; In-app Help</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
           <t>LAST — after final flows</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>PROGRAM TOTAL</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
-        <v>905</v>
-      </c>
-      <c r="D18" s="8" t="n">
-        <v>367</v>
-      </c>
-      <c r="F18" s="9" t="n">
-        <v>0.4033149171270718</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="C20" s="8" t="n">
+        <v>1035</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>439</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>0.4229951690821256</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>Key metrics</t>
         </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>Tasks total</t>
-        </is>
-      </c>
-      <c r="B21" s="11" t="n">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>Tasks Done</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="n">
-        <v>46</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>Tasks In Progress</t>
+          <t>Tasks total</t>
         </is>
       </c>
       <c r="B23" s="11" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>Tasks Pending</t>
+          <t>Tasks Done</t>
         </is>
       </c>
       <c r="B24" s="11" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>Tasks Blocked</t>
+          <t>Tasks In Progress</t>
         </is>
       </c>
       <c r="B25" s="11" t="n">
@@ -1093,68 +1128,88 @@
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>Estimated remaining effort (hrs)</t>
+          <t>Tasks Pending</t>
         </is>
       </c>
       <c r="B26" s="11" t="n">
-        <v>540</v>
+        <v>44</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>Estimated remaining duration (eng-days @6h)</t>
+          <t>Tasks Blocked</t>
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>67.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>Calendar hint (1 eng, critical path WP2→8)</t>
-        </is>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>~10–12 weeks after WP2 start (parallelize WP4/WP6)</t>
-        </is>
+          <t>Estimated remaining effort (hrs)</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="n">
+        <v>597.2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>PRs merged (commercial fork)</t>
-        </is>
-      </c>
-      <c r="B29" s="11" t="inlineStr">
-        <is>
-          <t>#1–#6</t>
-        </is>
+          <t>Estimated remaining duration (eng-days @6h)</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="n">
+        <v>74.90000000000001</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
+          <t>Calendar hint (1 eng, critical path WP2→8)</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>~10–12 weeks after WP2 start (parallelize WP4/WP6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>PRs merged (commercial fork)</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>#1–#6</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
           <t>Current package</t>
         </is>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>WP2 — Identity &amp; Microsoft Entra ID (kickoff in progress)</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="10" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
         <is>
           <t>Dependency graph (critical path)</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="60" customHeight="1">
-      <c r="A34" s="12" t="inlineStr">
+    <row r="36" ht="60" customHeight="1">
+      <c r="A36" s="12" t="inlineStr">
         <is>
           <t>WP0 → WP1 → WP-DEC(Model A) → WP2(Auth) → WP3(White-label) &amp; WP5(Connectors) → WP7(Packaging) → WP8(Onboarding)
 Parallel after foundations: WP4 (Backend map), WP6 (Benchmarks, needs hardware)
@@ -1164,8 +1219,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A36:G36"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A34:G34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1177,7 +1232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S93"/>
+  <dimension ref="A1:S101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5606,38 +5661,38 @@
     <row r="58" ht="75" customHeight="1">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.15</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>WP3 — Frontend Map + White-label</t>
+          <t>WP2b — Sharing &amp; Groups</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>WP3 kickoff</t>
+          <t>WP2b schema: groups + resource_grant + episode.notebook_id</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Purpose: start white-label work only after identity is on main.
-Steps: create wp-3-white-label; confirm Model A brand loads once at app startup (not per request).</t>
+          <t>Purpose: land the ACL data model without blocking on Entra directory sync.
+Steps: migration 28 — user_group (source local|entra, entra_group_oid), user_group_member, resource_grant (notebook|source × user|group × viewer|editor), episode.notebook_id for podcast inheritance.</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Branch</t>
-        </is>
-      </c>
-      <c r="F58" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G58" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>Migration 28 registered</t>
+        </is>
+      </c>
+      <c r="F58" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G58" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
@@ -5646,141 +5701,161 @@
         </is>
       </c>
       <c r="I58" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="J58" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="J58" s="17" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="K58" s="17" t="n"/>
+      <c r="K58" s="17" t="n">
+        <v>8</v>
+      </c>
       <c r="L58" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M58" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N58" s="19" t="n">
-        <v>46253</v>
+        <v>46240</v>
       </c>
       <c r="O58" s="19" t="n">
-        <v>46253</v>
-      </c>
-      <c r="P58" s="3" t="n"/>
+        <v>46240</v>
+      </c>
+      <c r="P58" s="19" t="n">
+        <v>46240</v>
+      </c>
       <c r="Q58" s="3" t="inlineStr">
         <is>
-          <t>Branch created after WP2 merge</t>
+          <t>Schema supports local groups now and Entra sync later without rewrite</t>
         </is>
       </c>
       <c r="R58" s="3" t="inlineStr">
         <is>
-          <t>Optional admin brand UI needs WP2 roles</t>
-        </is>
-      </c>
-      <c r="S58" s="3" t="inlineStr"/>
+          <t>entra_group_oid reserved; sync is follow-on 4.20</t>
+        </is>
+      </c>
+      <c r="S58" s="3" t="inlineStr">
+        <is>
+          <t>open_notebook/database/migrations/28.surrealql</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="75" customHeight="1">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.16</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>WP3 — Frontend Map + White-label</t>
+          <t>WP2b — Sharing &amp; Groups</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Produce docs/FRONTEND_MAP.md</t>
+          <t>Grant-aware access helpers + role matrix</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Purpose: make every future UI change locatable without archaeology.
-Steps: for each auth and dashboard route, document page → component tree, stores/hooks/API calls, shared layout, component catalog, and a where-do-I-change-X table.</t>
+          <t>Purpose: replace owner-only filters with owner OR user grant OR group grant; enforce viewer/editor matrix.
+Steps: extend api/ownership.py (access_where, source_access_where, effective_role, view/edit/delete asserts); editor cannot delete sources; viewer can chat/search/transform/play podcasts; stamp notebook_id on podcast generate.</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>docs/FRONTEND_MAP.md</t>
-        </is>
-      </c>
-      <c r="F59" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G59" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>api/ownership.py + router wiring</t>
+        </is>
+      </c>
+      <c r="F59" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G59" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.15</t>
         </is>
       </c>
       <c r="I59" s="17" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="J59" s="17" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="K59" s="17" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="K59" s="17" t="n">
+        <v>24</v>
+      </c>
       <c r="L59" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N59" s="19" t="n">
-        <v>46253</v>
+        <v>46240</v>
       </c>
       <c r="O59" s="19" t="n">
-        <v>46255</v>
-      </c>
-      <c r="P59" s="3" t="n"/>
+        <v>46240</v>
+      </c>
+      <c r="P59" s="19" t="n">
+        <v>46240</v>
+      </c>
       <c r="Q59" s="3" t="inlineStr">
         <is>
-          <t>Map covers every route with data flow + backend calls</t>
-        </is>
-      </c>
-      <c r="R59" s="3" t="inlineStr"/>
-      <c r="S59" s="3" t="inlineStr"/>
+          <t>Highest-wins roles; 404 when no access; 403 when visible but insufficient role</t>
+        </is>
+      </c>
+      <c r="R59" s="3" t="inlineStr">
+        <is>
+          <t>Locked matrix in docs/SHARING.md</t>
+        </is>
+      </c>
+      <c r="S59" s="3" t="inlineStr">
+        <is>
+          <t>api/ownership.py; tests/test_access_grants_unit.py</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="75" customHeight="1">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>4.17</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>WP3 — Frontend Map + White-label</t>
+          <t>WP2b — Sharing &amp; Groups</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>BrandConfig schema + loader</t>
+          <t>Groups + users picker + grants API</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Purpose: drive app name, logos, favicon, colours, font, and support URL from config so clients do not need a rebuild.
-Steps: define BrandConfig schema; load from BRAND_CONFIG_PATH or /config/brand at startup under Model A.</t>
+          <t>Purpose: admin-managed local groups; share/allocate via grant CRUD; picker = users who signed in at least once.
+Steps: /api/groups CRUD + members (admin mutate); GET /api/groups list for any auth user (share picker); GET /api/users; notebook/source grant endpoints (owner or admin).</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>BrandConfig type + loader</t>
-        </is>
-      </c>
-      <c r="F60" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+          <t>groups.py + grants.py routers</t>
+        </is>
+      </c>
+      <c r="F60" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G60" s="20" t="inlineStr">
@@ -5790,90 +5865,104 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.16</t>
         </is>
       </c>
       <c r="I60" s="17" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J60" s="17" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="K60" s="17" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="K60" s="17" t="n">
+        <v>16</v>
+      </c>
       <c r="L60" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M60" s="3" t="inlineStr">
         <is>
-          <t>Full-stack</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N60" s="19" t="n">
-        <v>46255</v>
+        <v>46240</v>
       </c>
       <c r="O60" s="19" t="n">
-        <v>46256</v>
-      </c>
-      <c r="P60" s="3" t="n"/>
+        <v>46240</v>
+      </c>
+      <c r="P60" s="19" t="n">
+        <v>46240</v>
+      </c>
       <c r="Q60" s="3" t="inlineStr">
         <is>
-          <t>Config loads without a rebuild</t>
-        </is>
-      </c>
-      <c r="R60" s="3" t="inlineStr"/>
-      <c r="S60" s="3" t="inlineStr"/>
+          <t>Owner can share; admin can allocate; non-members get 404</t>
+        </is>
+      </c>
+      <c r="R60" s="3" t="inlineStr">
+        <is>
+          <t>Full Entra directory picker deferred to 4.21</t>
+        </is>
+      </c>
+      <c r="S60" s="3" t="inlineStr">
+        <is>
+          <t>api/routers/groups.py; api/routers/grants.py</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="75" customHeight="1">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>4.18</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>WP3 — Frontend Map + White-label</t>
+          <t>WP2b — Sharing &amp; Groups</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Runtime theme injection (CSS variables)</t>
+          <t>Share dialog + Admin Groups UI + role gating</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Purpose: apply BrandConfig at runtime to CSS variables for light and dark themes.
-Steps: map colours to :root / dark variants; replace hardcoded title and /logo.svg; use the brand inventory in LICENSE_COMPLIANCE §8; demonstrate two brands from one build.</t>
+          <t>Purpose: ship the collaboration UX against the locked role matrix.
+Steps: ShareDialog on notebook/source; Settings → Groups (AdminOnly); hide/disable actions by access_role; i18n all locales.</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Runtime theming</t>
-        </is>
-      </c>
-      <c r="F61" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G61" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+          <t>Share UI + /settings/groups</t>
+        </is>
+      </c>
+      <c r="F61" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G61" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>4.17</t>
         </is>
       </c>
       <c r="I61" s="17" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="J61" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="K61" s="17" t="n"/>
+        <v>2.5</v>
+      </c>
+      <c r="K61" s="17" t="n">
+        <v>20</v>
+      </c>
       <c r="L61" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M61" s="3" t="inlineStr">
         <is>
@@ -5881,50 +5970,56 @@
         </is>
       </c>
       <c r="N61" s="19" t="n">
-        <v>46256</v>
+        <v>46240</v>
       </c>
       <c r="O61" s="19" t="n">
-        <v>46259</v>
-      </c>
-      <c r="P61" s="3" t="n"/>
+        <v>46240</v>
+      </c>
+      <c r="P61" s="19" t="n">
+        <v>46240</v>
+      </c>
       <c r="Q61" s="3" t="inlineStr">
         <is>
-          <t>Two visibly different brands from the same build; no code edit to rebrand</t>
+          <t>Viewer/editor/owner actions match SHARING.md; groups admin page works</t>
         </is>
       </c>
       <c r="R61" s="3" t="inlineStr"/>
-      <c r="S61" s="3" t="inlineStr"/>
+      <c r="S61" s="3" t="inlineStr">
+        <is>
+          <t>frontend/src/components/sharing/; settings/groups/</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="75" customHeight="1">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>5.4</t>
+          <t>4.19</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>WP3 — Frontend Map + White-label</t>
+          <t>WP2b — Sharing &amp; Groups</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>themes/ presets + add-client procedure</t>
+          <t>docs/SHARING.md + WP2b review stop</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Purpose: make “add a client theme” a documented drop-in of config + assets.
-Steps: ship at least two presets under themes/; write the operator procedure (no rebuild).</t>
+          <t>Purpose: document the sharing model and close WP2b without mixing WP3.
+Steps: write SHARING.md; AUTH.md pointer; update PDR-003; keep Entra sync / directory picker / public-link follow-ons as Pending WBS 4.20–4.22.</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>themes/ + docs procedure</t>
-        </is>
-      </c>
-      <c r="F62" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+          <t>docs/SHARING.md; branch ready for PR</t>
+        </is>
+      </c>
+      <c r="F62" s="25" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G62" s="16" t="inlineStr">
@@ -5934,64 +6029,76 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>4.18</t>
         </is>
       </c>
       <c r="I62" s="17" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J62" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="K62" s="17" t="n"/>
+        <v>0.75</v>
+      </c>
+      <c r="K62" s="17" t="n">
+        <v>4</v>
+      </c>
       <c r="L62" s="18" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="M62" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>Engineering Lead</t>
         </is>
       </c>
       <c r="N62" s="19" t="n">
-        <v>46259</v>
+        <v>46240</v>
       </c>
       <c r="O62" s="19" t="n">
-        <v>46260</v>
+        <v>46241</v>
       </c>
       <c r="P62" s="3" t="n"/>
       <c r="Q62" s="3" t="inlineStr">
         <is>
-          <t>Documented procedure produces two different brands from one build</t>
-        </is>
-      </c>
-      <c r="R62" s="3" t="inlineStr"/>
-      <c r="S62" s="3" t="inlineStr"/>
+          <t>SHARING.md complete; CI green; human review before merge; do not start WP3 on this branch</t>
+        </is>
+      </c>
+      <c r="R62" s="3" t="inlineStr">
+        <is>
+          <t>Follow-ons tracked in 4.20–4.22 — not blockers for WP2b merge</t>
+        </is>
+      </c>
+      <c r="S62" s="3" t="inlineStr">
+        <is>
+          <t>docs/SHARING.md; branch wp-2b-sharing</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="75" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>4.20</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>WP3 — Frontend Map + White-label</t>
+          <t>Carry-forward / Sharing Follow-through</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Optional admin BrandConfig UI</t>
+          <t>Entra ID group sync</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Purpose (optional): let admins edit BrandConfig live without redeploying.
-Steps: admin-only settings screen gated by WP2 roles; persist and hot-apply theme.</t>
+          <t>Purpose: make Entra security groups the primary group source (main goal after app-local groups).
+Why deferred: WP2b ships collaboration with local groups; Graph sync needs Group.Read.All (or equivalent), admin consent, membership sync job, and mapping Entra members → app users.
+Steps: (1) Graph app permissions + consent; (2) import/link Entra groups into user_group with source=entra and entra_group_oid; (3) sync membership into user_group_member; (4) refresh on schedule or webhook; (5) document in SHARING.md/AUTH.md.
+Schema already reserved in migration 28.</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Admin brand settings UI</t>
+          <t>Entra-backed groups with live membership</t>
         </is>
       </c>
       <c r="F63" s="22" t="inlineStr">
@@ -5999,21 +6106,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G63" s="24" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="G63" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>5.3,4.5</t>
+          <t>4.19</t>
         </is>
       </c>
       <c r="I63" s="17" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="J63" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K63" s="17" t="n"/>
       <c r="L63" s="18" t="n">
@@ -6021,53 +6128,54 @@
       </c>
       <c r="M63" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
-        </is>
-      </c>
-      <c r="N63" s="19" t="n">
-        <v>46260</v>
-      </c>
-      <c r="O63" s="19" t="n">
-        <v>46262</v>
-      </c>
+          <t>Backend Engineer</t>
+        </is>
+      </c>
+      <c r="N63" s="3" t="n"/>
+      <c r="O63" s="3" t="n"/>
       <c r="P63" s="3" t="n"/>
       <c r="Q63" s="3" t="inlineStr">
         <is>
-          <t>Admin can edit brand without redeploy (optional acceptance)</t>
+          <t>Admin can link an Entra group; membership changes in Entra reflect in ACL without re-sharing</t>
         </is>
       </c>
       <c r="R63" s="3" t="inlineStr">
         <is>
-          <t>Optional per master plan</t>
-        </is>
-      </c>
-      <c r="S63" s="3" t="inlineStr"/>
+          <t>Main post-WP2b goal for groups; do not rebuild ACL for this</t>
+        </is>
+      </c>
+      <c r="S63" s="3" t="inlineStr">
+        <is>
+          <t>user_group.source / entra_group_oid; docs/SHARING.md</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="75" customHeight="1">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>4.21</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>WP3 — Frontend Map + White-label</t>
+          <t>Carry-forward / Sharing Follow-through</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>WP3 verification + review stop</t>
+          <t>Full org directory user picker (Graph)</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Purpose: close white-label only when map + config branding acceptance criteria pass.
-Steps: verify ACs; PR; human review; do not mix WP5 on the same branch.</t>
+          <t>Purpose: let owners/admins pick any user in the Entra tenant, not only people who have already signed into the app.
+Why deferred: WP2b picker uses GET /api/users (JIT-provisioned DB rows only) to avoid Graph scopes and pending-grant edge cases.
+Steps: (1) Graph User.Read.All or equivalent search; (2) typeahead against tenant directory; (3) on grant to never-seen user, either JIT stub user or pending grant resolved at first login; (4) document privacy/consent.</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Merged WP3</t>
+          <t>Directory-backed share/group member picker</t>
         </is>
       </c>
       <c r="F64" s="22" t="inlineStr">
@@ -6082,14 +6190,14 @@
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>5.1,5.4</t>
+          <t>4.19</t>
         </is>
       </c>
       <c r="I64" s="17" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="J64" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K64" s="17" t="n"/>
       <c r="L64" s="18" t="n">
@@ -6097,49 +6205,56 @@
       </c>
       <c r="M64" s="3" t="inlineStr">
         <is>
-          <t>Engineering Lead</t>
-        </is>
-      </c>
-      <c r="N64" s="19" t="n">
-        <v>46262</v>
-      </c>
-      <c r="O64" s="19" t="n">
-        <v>46263</v>
-      </c>
+          <t>Full-stack</t>
+        </is>
+      </c>
+      <c r="N64" s="3" t="n"/>
+      <c r="O64" s="3" t="n"/>
       <c r="P64" s="3" t="n"/>
       <c r="Q64" s="3" t="inlineStr">
         <is>
-          <t>All WP3 acceptance criteria pass</t>
-        </is>
-      </c>
-      <c r="R64" s="3" t="inlineStr"/>
-      <c r="S64" s="3" t="inlineStr"/>
+          <t>Can share with a colleague who has never opened the app yet; first login attaches access</t>
+        </is>
+      </c>
+      <c r="R64" s="3" t="inlineStr">
+        <is>
+          <t>Pairs with 4.20; keep DB-user picker as fallback</t>
+        </is>
+      </c>
+      <c r="S64" s="3" t="inlineStr">
+        <is>
+          <t>GET /api/users today = signed-in only</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="75" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>4.22</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>WP4 — Backend/API Documentation</t>
+          <t>Carry-forward / Sharing Follow-through</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>WP4 kickoff (can parallel early)</t>
+          <t>Public links, editor reshare, ownership transfer</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Purpose: start the backend architecture map as documentation-only, low-risk work.
-Steps: create wp-4-backend-map; prefer starting after WP2 so auth docs match reality; can begin after WP0 if staffed in parallel.</t>
+          <t>Purpose: track three ACL product extensions explicitly out of WP2b.
+(1) Public / anyone-with-link sharing — rejected for enterprise Model A v1; revisit only with clear security model.
+(2) Editor reshare — Drive-like “editors can invite”; WP2b locks ACL manage to owner+admin only.
+(3) Ownership transfer — move user_id to another user without recreate.
+Steps: product decide each item; if approved, extend resource_grant / owner stamp + UI + docs; never enable public links by default.</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>Product decisions + optional follow-on features</t>
         </is>
       </c>
       <c r="F65" s="22" t="inlineStr">
@@ -6154,14 +6269,14 @@
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>4.19</t>
         </is>
       </c>
       <c r="I65" s="17" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="J65" s="17" t="n">
-        <v>0.25</v>
+        <v>2</v>
       </c>
       <c r="K65" s="17" t="n"/>
       <c r="L65" s="18" t="n">
@@ -6169,53 +6284,53 @@
       </c>
       <c r="M65" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
-        </is>
-      </c>
-      <c r="N65" s="19" t="n">
-        <v>46253</v>
-      </c>
-      <c r="O65" s="19" t="n">
-        <v>46253</v>
-      </c>
+          <t>Product / Engineer</t>
+        </is>
+      </c>
+      <c r="N65" s="3" t="n"/>
+      <c r="O65" s="3" t="n"/>
       <c r="P65" s="3" t="n"/>
       <c r="Q65" s="3" t="inlineStr">
         <is>
-          <t>Docs branch ready</t>
+          <t>Each item either shipped with tests/docs or explicitly rejected in SHARING.md</t>
         </is>
       </c>
       <c r="R65" s="3" t="inlineStr">
         <is>
-          <t>Better after WP2 for accurate auth sections</t>
-        </is>
-      </c>
-      <c r="S65" s="3" t="inlineStr"/>
+          <t>Not required for WP2b acceptance; do not sneak into WP3</t>
+        </is>
+      </c>
+      <c r="S65" s="3" t="inlineStr">
+        <is>
+          <t>docs/SHARING.md Deferred section</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="75" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>WP4 — Backend/API Documentation</t>
+          <t>WP3 — Frontend Map + White-label</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Router catalog (all endpoints)</t>
+          <t>WP3 kickoff</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Purpose: catalogue every HTTP endpoint with method, path, models, auth requirement, and service/domain call.
-Steps: walk all routers; document consistently; update after WP2 auth lands.</t>
+          <t>Purpose: start white-label work only after identity is on main.
+Steps: create wp-3-white-label; confirm Model A brand loads once at app startup (not per request).</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>BACKEND_MAP.md routers section</t>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F66" s="22" t="inlineStr">
@@ -6223,21 +6338,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G66" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G66" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>4.19</t>
         </is>
       </c>
       <c r="I66" s="17" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="J66" s="17" t="n">
-        <v>2</v>
+        <v>0.25</v>
       </c>
       <c r="K66" s="17" t="n"/>
       <c r="L66" s="18" t="n">
@@ -6245,49 +6360,53 @@
       </c>
       <c r="M66" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N66" s="19" t="n">
         <v>46253</v>
       </c>
       <c r="O66" s="19" t="n">
-        <v>46255</v>
+        <v>46253</v>
       </c>
       <c r="P66" s="3" t="n"/>
       <c r="Q66" s="3" t="inlineStr">
         <is>
-          <t>Every endpoint documented with auth + models</t>
-        </is>
-      </c>
-      <c r="R66" s="3" t="inlineStr"/>
+          <t>Branch created after WP2b merge (or after WP2 if WP2b still open — prefer after 4.19)</t>
+        </is>
+      </c>
+      <c r="R66" s="3" t="inlineStr">
+        <is>
+          <t>Optional admin brand UI needs WP2 roles; do not mix with wp-2b-sharing</t>
+        </is>
+      </c>
       <c r="S66" s="3" t="inlineStr"/>
     </row>
     <row r="67" ht="75" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>WP4 — Backend/API Documentation</t>
+          <t>WP3 — Frontend Map + White-label</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Domain model + graph + data layer maps</t>
+          <t>Produce docs/FRONTEND_MAP.md</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Purpose: document ObjectModel patterns, LangGraph flows, repository usage, migrations, and SurrealDB features in use.
-Steps: catalogue models/relationships; map each graph’s inputs/steps/outputs; explain repository call-site pattern and migrations.</t>
+          <t>Purpose: make every future UI change locatable without archaeology.
+Steps: for each auth and dashboard route, document page → component tree, stores/hooks/API calls, shared layout, component catalog, and a where-do-I-change-X table.</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>BACKEND_MAP.md domain/graphs/data</t>
+          <t>docs/FRONTEND_MAP.md</t>
         </is>
       </c>
       <c r="F67" s="22" t="inlineStr">
@@ -6295,21 +6414,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G67" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G67" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="I67" s="17" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="J67" s="17" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="K67" s="17" t="n"/>
       <c r="L67" s="18" t="n">
@@ -6317,19 +6436,19 @@
       </c>
       <c r="M67" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N67" s="19" t="n">
+        <v>46253</v>
+      </c>
+      <c r="O67" s="19" t="n">
         <v>46255</v>
-      </c>
-      <c r="O67" s="19" t="n">
-        <v>46259</v>
       </c>
       <c r="P67" s="3" t="n"/>
       <c r="Q67" s="3" t="inlineStr">
         <is>
-          <t>Every domain model and graph documented</t>
+          <t>Map covers every route with data flow + backend calls</t>
         </is>
       </c>
       <c r="R67" s="3" t="inlineStr"/>
@@ -6338,28 +6457,28 @@
     <row r="68" ht="75" customHeight="1">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>6.3</t>
+          <t>5.2</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>WP4 — Backend/API Documentation</t>
+          <t>WP3 — Frontend Map + White-label</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Jobs, config/secrets, how-to playbooks</t>
+          <t>BrandConfig schema + loader</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Purpose: finish the operator/engineer map with jobs, env vars, and five how-to-add playbooks.
-Steps: document surreal-commands; env/secrets; playbooks for endpoint, model+migration, provider, job, source type; reconcile with existing change-playbooks.md.</t>
+          <t>Purpose: drive app name, logos, favicon, colours, font, and support URL from config so clients do not need a rebuild.
+Steps: define BrandConfig schema; load from BRAND_CONFIG_PATH or /config/brand at startup under Model A.</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>BACKEND_MAP.md complete</t>
+          <t>BrandConfig type + loader</t>
         </is>
       </c>
       <c r="F68" s="22" t="inlineStr">
@@ -6367,14 +6486,14 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G68" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G68" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="I68" s="17" t="n">
@@ -6389,19 +6508,19 @@
       </c>
       <c r="M68" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Full-stack</t>
         </is>
       </c>
       <c r="N68" s="19" t="n">
-        <v>46259</v>
+        <v>46255</v>
       </c>
       <c r="O68" s="19" t="n">
-        <v>46260</v>
+        <v>46256</v>
       </c>
       <c r="P68" s="3" t="n"/>
       <c r="Q68" s="3" t="inlineStr">
         <is>
-          <t>Five how-to playbooks present and accurate</t>
+          <t>Config loads without a rebuild</t>
         </is>
       </c>
       <c r="R68" s="3" t="inlineStr"/>
@@ -6410,28 +6529,28 @@
     <row r="69" ht="75" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>6.4</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>WP4 — Backend/API Documentation</t>
+          <t>WP3 — Frontend Map + White-label</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>WP4 review stop</t>
+          <t>Runtime theme injection (CSS variables)</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Purpose: peer-review the map for accuracy and merge.
-Steps: review against live code; fix gaps; merge; confirm a new engineer can locate changes using only BACKEND_MAP.</t>
+          <t>Purpose: apply BrandConfig at runtime to CSS variables for light and dark themes.
+Steps: map colours to :root / dark variants; replace hardcoded title and /logo.svg; use the brand inventory in LICENSE_COMPLIANCE §8; demonstrate two brands from one build.</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>docs/BACKEND_MAP.md on main</t>
+          <t>Runtime theming</t>
         </is>
       </c>
       <c r="F69" s="22" t="inlineStr">
@@ -6439,21 +6558,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G69" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G69" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>6.3</t>
+          <t>5.2</t>
         </is>
       </c>
       <c r="I69" s="17" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="J69" s="17" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="K69" s="17" t="n"/>
       <c r="L69" s="18" t="n">
@@ -6461,19 +6580,19 @@
       </c>
       <c r="M69" s="3" t="inlineStr">
         <is>
-          <t>Engineering Lead</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N69" s="19" t="n">
-        <v>46260</v>
+        <v>46256</v>
       </c>
       <c r="O69" s="19" t="n">
-        <v>46261</v>
+        <v>46259</v>
       </c>
       <c r="P69" s="3" t="n"/>
       <c r="Q69" s="3" t="inlineStr">
         <is>
-          <t>New engineer can locate changes using only this doc</t>
+          <t>Two visibly different brands from the same build; no code edit to rebrand</t>
         </is>
       </c>
       <c r="R69" s="3" t="inlineStr"/>
@@ -6482,28 +6601,28 @@
     <row r="70" ht="75" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>7.0</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>WP5 — External Source Connectors</t>
+          <t>WP3 — Frontend Map + White-label</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>WP5 kickoff</t>
+          <t>themes/ presets + add-client procedure</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Purpose: design connectors that feed the existing ingestion pipeline instead of reinventing extraction.
-Steps: create wp-5-connectors; draft SourceConnector interface; confirm hard dependency on WP2 for per-user OAuth tokens.</t>
+          <t>Purpose: make “add a client theme” a documented drop-in of config + assets.
+Steps: ship at least two presets under themes/; write the operator procedure (no rebuild).</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Branch + design note</t>
+          <t>themes/ + docs procedure</t>
         </is>
       </c>
       <c r="F70" s="22" t="inlineStr">
@@ -6518,14 +6637,14 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>4.10</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="I70" s="17" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J70" s="17" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K70" s="17" t="n"/>
       <c r="L70" s="18" t="n">
@@ -6533,53 +6652,49 @@
       </c>
       <c r="M70" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N70" s="19" t="n">
-        <v>46266</v>
+        <v>46259</v>
       </c>
       <c r="O70" s="19" t="n">
-        <v>46266</v>
+        <v>46260</v>
       </c>
       <c r="P70" s="3" t="n"/>
       <c r="Q70" s="3" t="inlineStr">
         <is>
-          <t>Design reuses content-core + graphs/source.py</t>
-        </is>
-      </c>
-      <c r="R70" s="3" t="inlineStr">
-        <is>
-          <t>Blocked until WP2 users/tokens exist</t>
-        </is>
-      </c>
+          <t>Documented procedure produces two different brands from one build</t>
+        </is>
+      </c>
+      <c r="R70" s="3" t="inlineStr"/>
       <c r="S70" s="3" t="inlineStr"/>
     </row>
     <row r="71" ht="75" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>WP5 — External Source Connectors</t>
+          <t>WP3 — Frontend Map + White-label</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>SourceConnector interface + bulk job fan-out</t>
+          <t>Optional admin BrandConfig UI</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Purpose: one “add location” action becomes N document jobs with per-doc progress and partial failure tolerance.
-Steps: define authenticate/list_documents/fetch_document; extend source_commands for fan-out; ensure one bad file does not abort the batch.</t>
+          <t>Purpose (optional): let admins edit BrandConfig live without redeploying.
+Steps: admin-only settings screen gated by WP2 roles; persist and hot-apply theme.</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Connector API + bulk command</t>
+          <t>Admin brand settings UI</t>
         </is>
       </c>
       <c r="F71" s="22" t="inlineStr">
@@ -6587,21 +6702,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G71" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G71" s="24" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>7.0</t>
+          <t>5.3,4.5</t>
         </is>
       </c>
       <c r="I71" s="17" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="J71" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K71" s="17" t="n"/>
       <c r="L71" s="18" t="n">
@@ -6609,49 +6724,53 @@
       </c>
       <c r="M71" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N71" s="19" t="n">
-        <v>46266</v>
+        <v>46260</v>
       </c>
       <c r="O71" s="19" t="n">
-        <v>46269</v>
+        <v>46262</v>
       </c>
       <c r="P71" s="3" t="n"/>
       <c r="Q71" s="3" t="inlineStr">
         <is>
-          <t>Single failure does not abort batch; progress per document</t>
-        </is>
-      </c>
-      <c r="R71" s="3" t="inlineStr"/>
+          <t>Admin can edit brand without redeploy (optional acceptance)</t>
+        </is>
+      </c>
+      <c r="R71" s="3" t="inlineStr">
+        <is>
+          <t>Optional per master plan</t>
+        </is>
+      </c>
       <c r="S71" s="3" t="inlineStr"/>
     </row>
     <row r="72" ht="75" customHeight="1">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>WP5 — External Source Connectors</t>
+          <t>WP3 — Frontend Map + White-label</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>SharePoint connector (Microsoft Graph)</t>
+          <t>WP3 verification + review stop</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Purpose: let an Entra-signed-in user pull an entire SharePoint folder into chat-able sources.
-Steps: OAuth on behalf of the user; least-privilege Sites/Files read scopes; enumerate folder; download supported files into existing ingestion; document admin consent.</t>
+          <t>Purpose: close white-label only when map + config branding acceptance criteria pass.
+Steps: verify ACs; PR; human review; do not mix WP5 on the same branch.</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>SharePointConnector</t>
+          <t>Merged WP3</t>
         </is>
       </c>
       <c r="F72" s="22" t="inlineStr">
@@ -6659,21 +6778,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G72" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G72" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>7.1,4.7</t>
+          <t>5.1,5.4</t>
         </is>
       </c>
       <c r="I72" s="17" t="n">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="J72" s="17" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K72" s="17" t="n"/>
       <c r="L72" s="18" t="n">
@@ -6681,19 +6800,19 @@
       </c>
       <c r="M72" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Engineering Lead</t>
         </is>
       </c>
       <c r="N72" s="19" t="n">
-        <v>46269</v>
+        <v>46262</v>
       </c>
       <c r="O72" s="19" t="n">
-        <v>46275</v>
+        <v>46263</v>
       </c>
       <c r="P72" s="3" t="n"/>
       <c r="Q72" s="3" t="inlineStr">
         <is>
-          <t>User connects SharePoint, picks folder, pulls all supported docs</t>
+          <t>All WP3 acceptance criteria pass</t>
         </is>
       </c>
       <c r="R72" s="3" t="inlineStr"/>
@@ -6702,28 +6821,28 @@
     <row r="73" ht="75" customHeight="1">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>WP5 — External Source Connectors</t>
+          <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Generic DMS / multi-doc link connector</t>
+          <t>WP4 kickoff (can parallel early)</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Purpose: support folder URLs / IDs that resolve to many documents, with an extension point for other DMS systems.
-Steps: implement base multi-doc connector; keep the SourceConnector interface as the only required surface for new connectors.</t>
+          <t>Purpose: start the backend architecture map as documentation-only, low-risk work.
+Steps: create wp-4-backend-map; prefer starting after WP2 so auth docs match reality; can begin after WP0 if staffed in parallel.</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Generic multi-doc connector</t>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F73" s="22" t="inlineStr">
@@ -6731,21 +6850,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G73" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G73" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="I73" s="17" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="J73" s="17" t="n">
-        <v>2</v>
+        <v>0.25</v>
       </c>
       <c r="K73" s="17" t="n"/>
       <c r="L73" s="18" t="n">
@@ -6757,45 +6876,49 @@
         </is>
       </c>
       <c r="N73" s="19" t="n">
-        <v>46273</v>
+        <v>46253</v>
       </c>
       <c r="O73" s="19" t="n">
-        <v>46275</v>
+        <v>46253</v>
       </c>
       <c r="P73" s="3" t="n"/>
       <c r="Q73" s="3" t="inlineStr">
         <is>
-          <t>New connector = implement interface only</t>
-        </is>
-      </c>
-      <c r="R73" s="3" t="inlineStr"/>
+          <t>Docs branch ready</t>
+        </is>
+      </c>
+      <c r="R73" s="3" t="inlineStr">
+        <is>
+          <t>Better after WP2 for accurate auth sections</t>
+        </is>
+      </c>
       <c r="S73" s="3" t="inlineStr"/>
     </row>
     <row r="74" ht="75" customHeight="1">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>7.4</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>WP5 — External Source Connectors</t>
+          <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Encrypted per-user token storage</t>
+          <t>Router catalog (all endpoints)</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Purpose: store connector OAuth tokens encrypted per user using existing encryption-key infrastructure.
-Steps: persist tokens encrypted; never share across users; respect source-system permissions (never fetch what the user cannot access).</t>
+          <t>Purpose: catalogue every HTTP endpoint with method, path, models, auth requirement, and service/domain call.
+Steps: walk all routers; document consistently; update after WP2 auth lands.</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>Encrypted token store</t>
+          <t>BACKEND_MAP.md routers section</t>
         </is>
       </c>
       <c r="F74" s="22" t="inlineStr">
@@ -6803,21 +6926,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G74" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G74" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>7.2,2.8</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="I74" s="17" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J74" s="17" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="K74" s="17" t="n"/>
       <c r="L74" s="18" t="n">
@@ -6829,15 +6952,15 @@
         </is>
       </c>
       <c r="N74" s="19" t="n">
-        <v>46275</v>
+        <v>46253</v>
       </c>
       <c r="O74" s="19" t="n">
-        <v>46276</v>
+        <v>46255</v>
       </c>
       <c r="P74" s="3" t="n"/>
       <c r="Q74" s="3" t="inlineStr">
         <is>
-          <t>Tokens encrypted per user; no cross-user leak</t>
+          <t>Every endpoint documented with auth + models</t>
         </is>
       </c>
       <c r="R74" s="3" t="inlineStr"/>
@@ -6846,28 +6969,28 @@
     <row r="75" ht="75" customHeight="1">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>WP5 — External Source Connectors</t>
+          <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Frontend: Add from SharePoint / Link flow</t>
+          <t>Domain model + graph + data layer maps</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Purpose: ship the operator UX for connect → folder pick → select → progress, then chat across the pulled set.
-Steps: add sources steps UI; show per-doc progress; ensure i18n for all locales; group pulled docs for chat/search.</t>
+          <t>Purpose: document ObjectModel patterns, LangGraph flows, repository usage, migrations, and SurrealDB features in use.
+Steps: catalogue models/relationships; map each graph’s inputs/steps/outputs; explain repository call-site pattern and migrations.</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Sources UI flow</t>
+          <t>BACKEND_MAP.md domain/graphs/data</t>
         </is>
       </c>
       <c r="F75" s="22" t="inlineStr">
@@ -6875,21 +6998,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G75" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G75" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>7.2,7.3</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="I75" s="17" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="J75" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K75" s="17" t="n"/>
       <c r="L75" s="18" t="n">
@@ -6897,53 +7020,49 @@
       </c>
       <c r="M75" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N75" s="19" t="n">
-        <v>46276</v>
+        <v>46255</v>
       </c>
       <c r="O75" s="19" t="n">
-        <v>46281</v>
+        <v>46259</v>
       </c>
       <c r="P75" s="3" t="n"/>
       <c r="Q75" s="3" t="inlineStr">
         <is>
-          <t>User can chat across the whole pulled set</t>
-        </is>
-      </c>
-      <c r="R75" s="3" t="inlineStr">
-        <is>
-          <t>i18n required for all locales</t>
-        </is>
-      </c>
+          <t>Every domain model and graph documented</t>
+        </is>
+      </c>
+      <c r="R75" s="3" t="inlineStr"/>
       <c r="S75" s="3" t="inlineStr"/>
     </row>
     <row r="76" ht="75" customHeight="1">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>7.6</t>
+          <t>6.3</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>WP5 — External Source Connectors</t>
+          <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>docs/CONNECTORS.md + WP5 review</t>
+          <t>Jobs, config/secrets, how-to playbooks</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Purpose: document Entra scopes/consent and how to add a connector; close WP5 on acceptance criteria.
-Steps: write CONNECTORS.md; verify ACs; PR; human review stop.</t>
+          <t>Purpose: finish the operator/engineer map with jobs, env vars, and five how-to-add playbooks.
+Steps: document surreal-commands; env/secrets; playbooks for endpoint, model+migration, provider, job, source type; reconcile with existing change-playbooks.md.</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>docs/CONNECTORS.md; merged WP5</t>
+          <t>BACKEND_MAP.md complete</t>
         </is>
       </c>
       <c r="F76" s="22" t="inlineStr">
@@ -6951,21 +7070,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G76" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G76" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>7.4,7.5</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="I76" s="17" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J76" s="17" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="K76" s="17" t="n"/>
       <c r="L76" s="18" t="n">
@@ -6973,19 +7092,19 @@
       </c>
       <c r="M76" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N76" s="19" t="n">
-        <v>46281</v>
+        <v>46259</v>
       </c>
       <c r="O76" s="19" t="n">
-        <v>46282</v>
+        <v>46260</v>
       </c>
       <c r="P76" s="3" t="n"/>
       <c r="Q76" s="3" t="inlineStr">
         <is>
-          <t>All WP5 acceptance criteria pass</t>
+          <t>Five how-to playbooks present and accurate</t>
         </is>
       </c>
       <c r="R76" s="3" t="inlineStr"/>
@@ -6994,28 +7113,28 @@
     <row r="77" ht="75" customHeight="1">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>WP6 — Doc Processing Benchmarks</t>
+          <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>WP6 kickoff + enumerate supported types</t>
+          <t>WP4 review stop</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Purpose: list what content-core actually supports today and what needs work (OCR, EPUB, upload HTML, etc.).
-Steps: inventory from real code/config; note gaps; create wp-6-benchmarks. Can run after WP0; needs target hardware for later measurement tasks.</t>
+          <t>Purpose: peer-review the map for accuracy and merge.
+Steps: review against live code; fix gaps; merge; confirm a new engineer can locate changes using only BACKEND_MAP.</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Type inventory</t>
+          <t>docs/BACKEND_MAP.md on main</t>
         </is>
       </c>
       <c r="F77" s="22" t="inlineStr">
@@ -7030,14 +7149,14 @@
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>6.3</t>
         </is>
       </c>
       <c r="I77" s="17" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J77" s="17" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="K77" s="17" t="n"/>
       <c r="L77" s="18" t="n">
@@ -7045,53 +7164,49 @@
       </c>
       <c r="M77" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Engineering Lead</t>
         </is>
       </c>
       <c r="N77" s="19" t="n">
-        <v>46266</v>
+        <v>46260</v>
       </c>
       <c r="O77" s="19" t="n">
-        <v>46267</v>
+        <v>46261</v>
       </c>
       <c r="P77" s="3" t="n"/>
       <c r="Q77" s="3" t="inlineStr">
         <is>
-          <t>Supported types documented from real code</t>
-        </is>
-      </c>
-      <c r="R77" s="3" t="inlineStr">
-        <is>
-          <t>No guessed client-facing numbers</t>
-        </is>
-      </c>
+          <t>New engineer can locate changes using only this doc</t>
+        </is>
+      </c>
+      <c r="R77" s="3" t="inlineStr"/>
       <c r="S77" s="3" t="inlineStr"/>
     </row>
     <row r="78" ht="75" customHeight="1">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.0</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>WP6 — Doc Processing Benchmarks</t>
+          <t>WP5 — External Source Connectors</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Build /benchmarks/ harness</t>
+          <t>WP5 kickoff</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Purpose: produce repeatable measured metrics — not estimates — for ingestion, extraction, embedding, memory, and search/chat latency.
-Steps: build parameterized harness under /benchmarks/; output machine-readable reports.</t>
+          <t>Purpose: design connectors that feed the existing ingestion pipeline instead of reinventing extraction.
+Steps: create wp-5-connectors; draft SourceConnector interface; confirm hard dependency on WP2 for per-user OAuth tokens.</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>/benchmarks/ harness</t>
+          <t>Branch + design note</t>
         </is>
       </c>
       <c r="F78" s="22" t="inlineStr">
@@ -7106,14 +7221,14 @@
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>4.10</t>
         </is>
       </c>
       <c r="I78" s="17" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="J78" s="17" t="n">
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="K78" s="17" t="n"/>
       <c r="L78" s="18" t="n">
@@ -7125,45 +7240,49 @@
         </is>
       </c>
       <c r="N78" s="19" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="O78" s="19" t="n">
-        <v>46270</v>
+        <v>46266</v>
       </c>
       <c r="P78" s="3" t="n"/>
       <c r="Q78" s="3" t="inlineStr">
         <is>
-          <t>Harness runs repeatably and outputs a metrics report</t>
-        </is>
-      </c>
-      <c r="R78" s="3" t="inlineStr"/>
+          <t>Design reuses content-core + graphs/source.py</t>
+        </is>
+      </c>
+      <c r="R78" s="3" t="inlineStr">
+        <is>
+          <t>Blocked until WP2 users/tokens exist</t>
+        </is>
+      </c>
       <c r="S78" s="3" t="inlineStr"/>
     </row>
     <row r="79" ht="75" customHeight="1">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>WP6 — Doc Processing Benchmarks</t>
+          <t>WP5 — External Source Connectors</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Assemble representative corpus</t>
+          <t>SourceConnector interface + bulk job fan-out</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Purpose: find empirical slowdown/failure points across sizes and types.
-Steps: assemble small/medium/large/very-large docs plus scanned PDF, audio, and web page; ensure corpus licensing is clean for redistribution in-repo if needed.</t>
+          <t>Purpose: one “add location” action becomes N document jobs with per-doc progress and partial failure tolerance.
+Steps: define authenticate/list_documents/fetch_document; extend source_commands for fan-out; ensure one bad file does not abort the batch.</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Fixed corpus under benchmarks/</t>
+          <t>Connector API + bulk command</t>
         </is>
       </c>
       <c r="F79" s="22" t="inlineStr">
@@ -7171,21 +7290,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G79" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G79" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.0</t>
         </is>
       </c>
       <c r="I79" s="17" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="J79" s="17" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="K79" s="17" t="n"/>
       <c r="L79" s="18" t="n">
@@ -7193,19 +7312,19 @@
       </c>
       <c r="M79" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N79" s="19" t="n">
-        <v>46270</v>
+        <v>46266</v>
       </c>
       <c r="O79" s="19" t="n">
-        <v>46273</v>
+        <v>46269</v>
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="inlineStr">
         <is>
-          <t>Corpus covers the size/type matrix</t>
+          <t>Single failure does not abort batch; progress per document</t>
         </is>
       </c>
       <c r="R79" s="3" t="inlineStr"/>
@@ -7214,28 +7333,28 @@
     <row r="80" ht="75" customHeight="1">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>WP6 — Doc Processing Benchmarks</t>
+          <t>WP5 — External Source Connectors</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Define accuracy methodology</t>
+          <t>SharePoint connector (Microsoft Graph)</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Purpose: define how accuracy is measured so client claims are defensible.
-Steps: specify extraction fidelity, retrieval relevance (labeled Q&amp;A), and chat groundedness methods; report per model tier.</t>
+          <t>Purpose: let an Entra-signed-in user pull an entire SharePoint folder into chat-able sources.
+Steps: OAuth on behalf of the user; least-privilege Sites/Files read scopes; enumerate folder; download supported files into existing ingestion; document admin consent.</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>Accuracy method doc section</t>
+          <t>SharePointConnector</t>
         </is>
       </c>
       <c r="F80" s="22" t="inlineStr">
@@ -7243,21 +7362,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G80" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G80" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.1,4.7</t>
         </is>
       </c>
       <c r="I80" s="17" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="J80" s="17" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K80" s="17" t="n"/>
       <c r="L80" s="18" t="n">
@@ -7265,19 +7384,19 @@
       </c>
       <c r="M80" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N80" s="19" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="O80" s="19" t="n">
-        <v>46273</v>
+        <v>46275</v>
       </c>
       <c r="P80" s="3" t="n"/>
       <c r="Q80" s="3" t="inlineStr">
         <is>
-          <t>Accuracy reported as method + numbers</t>
+          <t>User connects SharePoint, picks folder, pulls all supported docs</t>
         </is>
       </c>
       <c r="R80" s="3" t="inlineStr"/>
@@ -7286,28 +7405,28 @@
     <row r="81" ht="75" customHeight="1">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>WP6 — Doc Processing Benchmarks</t>
+          <t>WP5 — External Source Connectors</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Run ≥2 hardware profiles</t>
+          <t>Generic DMS / multi-doc link connector</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Purpose: gather real numbers on bare-minimum and recommended hardware.
-Steps: run harness on both profiles; record figures; note local-model vs API-provider resource differences. Requires access to target hardware.</t>
+          <t>Purpose: support folder URLs / IDs that resolve to many documents, with an extension point for other DMS systems.
+Steps: implement base multi-doc connector; keep the SourceConnector interface as the only required surface for new connectors.</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Raw results JSON/CSV</t>
+          <t>Generic multi-doc connector</t>
         </is>
       </c>
       <c r="F81" s="22" t="inlineStr">
@@ -7315,21 +7434,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G81" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G81" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>8.2,8.3</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="I81" s="17" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="J81" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K81" s="17" t="n"/>
       <c r="L81" s="18" t="n">
@@ -7337,53 +7456,49 @@
       </c>
       <c r="M81" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N81" s="19" t="n">
         <v>46273</v>
       </c>
       <c r="O81" s="19" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="P81" s="3" t="n"/>
       <c r="Q81" s="3" t="inlineStr">
         <is>
-          <t>Real measured numbers for both profiles</t>
-        </is>
-      </c>
-      <c r="R81" s="3" t="inlineStr">
-        <is>
-          <t>Hardware access is a dependency</t>
-        </is>
-      </c>
+          <t>New connector = implement interface only</t>
+        </is>
+      </c>
+      <c r="R81" s="3" t="inlineStr"/>
       <c r="S81" s="3" t="inlineStr"/>
     </row>
     <row r="82" ht="75" customHeight="1">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>7.4</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>WP6 — Doc Processing Benchmarks</t>
+          <t>WP5 — External Source Connectors</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>docs/PERFORMANCE_AND_SIZING.md + review</t>
+          <t>Encrypted per-user token storage</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Purpose: publish client-facing sizing guidance backed only by harness output.
-Steps: write types, limits, times, accuracy, min vs recommended hardware; peer review; merge.</t>
+          <t>Purpose: store connector OAuth tokens encrypted per user using existing encryption-key infrastructure.
+Steps: persist tokens encrypted; never share across users; respect source-system permissions (never fetch what the user cannot access).</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>docs/PERFORMANCE_AND_SIZING.md</t>
+          <t>Encrypted token store</t>
         </is>
       </c>
       <c r="F82" s="22" t="inlineStr">
@@ -7391,21 +7506,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G82" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G82" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>7.2,2.8</t>
         </is>
       </c>
       <c r="I82" s="17" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J82" s="17" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="K82" s="17" t="n"/>
       <c r="L82" s="18" t="n">
@@ -7413,19 +7528,19 @@
       </c>
       <c r="M82" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N82" s="19" t="n">
+        <v>46275</v>
+      </c>
+      <c r="O82" s="19" t="n">
         <v>46276</v>
-      </c>
-      <c r="O82" s="19" t="n">
-        <v>46277</v>
       </c>
       <c r="P82" s="3" t="n"/>
       <c r="Q82" s="3" t="inlineStr">
         <is>
-          <t>Doc contains measured numbers only</t>
+          <t>Tokens encrypted per user; no cross-user leak</t>
         </is>
       </c>
       <c r="R82" s="3" t="inlineStr"/>
@@ -7434,28 +7549,28 @@
     <row r="83" ht="75" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>WP7 — Cross-platform Packaging</t>
+          <t>WP5 — External Source Connectors</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>WP7 kickoff</t>
+          <t>Frontend: Add from SharePoint / Link flow</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Purpose: package the real authenticated + branded app, not the pre-WP2 password prototype.
-Steps: create wp-7-packaging only after WP2 and WP3 are on main.</t>
+          <t>Purpose: ship the operator UX for connect → folder pick → select → progress, then chat across the pulled set.
+Steps: add sources steps UI; show per-doc progress; ensure i18n for all locales; group pulled docs for chat/search.</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>Sources UI flow</t>
         </is>
       </c>
       <c r="F83" s="22" t="inlineStr">
@@ -7470,14 +7585,14 @@
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>5.6,4.10</t>
+          <t>7.2,7.3</t>
         </is>
       </c>
       <c r="I83" s="17" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="J83" s="17" t="n">
-        <v>0.25</v>
+        <v>3</v>
       </c>
       <c r="K83" s="17" t="n"/>
       <c r="L83" s="18" t="n">
@@ -7485,49 +7600,53 @@
       </c>
       <c r="M83" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N83" s="19" t="n">
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="O83" s="19" t="n">
-        <v>46283</v>
+        <v>46281</v>
       </c>
       <c r="P83" s="3" t="n"/>
       <c r="Q83" s="3" t="inlineStr">
         <is>
-          <t>Starts only after branded + authenticated app exists</t>
-        </is>
-      </c>
-      <c r="R83" s="3" t="inlineStr"/>
+          <t>User can chat across the whole pulled set</t>
+        </is>
+      </c>
+      <c r="R83" s="3" t="inlineStr">
+        <is>
+          <t>i18n required for all locales</t>
+        </is>
+      </c>
       <c r="S83" s="3" t="inlineStr"/>
     </row>
     <row r="84" ht="75" customHeight="1">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>7.6</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>WP7 — Cross-platform Packaging</t>
+          <t>WP5 — External Source Connectors</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Verify Docker Compose on Windows + Linux</t>
+          <t>docs/CONNECTORS.md + WP5 review</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Purpose: make containers the recommended identical path on both OSes.
-Steps: verify docker-compose and Dockerfile.single on Docker Desktop/WSL2 and Linux; document as primary deploy path.</t>
+          <t>Purpose: document Entra scopes/consent and how to add a connector; close WP5 on acceptance criteria.
+Steps: write CONNECTORS.md; verify ACs; PR; human review stop.</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>Verified container deploy</t>
+          <t>docs/CONNECTORS.md; merged WP5</t>
         </is>
       </c>
       <c r="F84" s="22" t="inlineStr">
@@ -7535,21 +7654,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G84" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G84" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>7.4,7.5</t>
         </is>
       </c>
       <c r="I84" s="17" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="J84" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K84" s="17" t="n"/>
       <c r="L84" s="18" t="n">
@@ -7557,19 +7676,19 @@
       </c>
       <c r="M84" s="3" t="inlineStr">
         <is>
-          <t>DevOps / Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N84" s="19" t="n">
-        <v>46283</v>
+        <v>46281</v>
       </c>
       <c r="O84" s="19" t="n">
-        <v>46287</v>
+        <v>46282</v>
       </c>
       <c r="P84" s="3" t="n"/>
       <c r="Q84" s="3" t="inlineStr">
         <is>
-          <t>Container deployment verified on both OSes</t>
+          <t>All WP5 acceptance criteria pass</t>
         </is>
       </c>
       <c r="R84" s="3" t="inlineStr"/>
@@ -7578,28 +7697,28 @@
     <row r="85" ht="75" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>WP7 — Cross-platform Packaging</t>
+          <t>WP6 — Doc Processing Benchmarks</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Native Linux install path (systemd)</t>
+          <t>WP6 kickoff + enumerate supported types</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Purpose: support customers who refuse containers.
-Steps: systemd units + install script; document dependencies for common distros; verify on at least one distro.</t>
+          <t>Purpose: list what content-core actually supports today and what needs work (OCR, EPUB, upload HTML, etc.).
+Steps: inventory from real code/config; note gaps; create wp-6-benchmarks. Can run after WP0; needs target hardware for later measurement tasks.</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Linux native docs + scripts</t>
+          <t>Type inventory</t>
         </is>
       </c>
       <c r="F85" s="22" t="inlineStr">
@@ -7614,14 +7733,14 @@
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="I85" s="17" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="J85" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K85" s="17" t="n"/>
       <c r="L85" s="18" t="n">
@@ -7629,49 +7748,53 @@
       </c>
       <c r="M85" s="3" t="inlineStr">
         <is>
-          <t>DevOps / Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N85" s="19" t="n">
-        <v>46287</v>
+        <v>46266</v>
       </c>
       <c r="O85" s="19" t="n">
-        <v>46289</v>
+        <v>46267</v>
       </c>
       <c r="P85" s="3" t="n"/>
       <c r="Q85" s="3" t="inlineStr">
         <is>
-          <t>Verified on ≥1 Linux distro</t>
-        </is>
-      </c>
-      <c r="R85" s="3" t="inlineStr"/>
+          <t>Supported types documented from real code</t>
+        </is>
+      </c>
+      <c r="R85" s="3" t="inlineStr">
+        <is>
+          <t>No guessed client-facing numbers</t>
+        </is>
+      </c>
       <c r="S85" s="3" t="inlineStr"/>
     </row>
     <row r="86" ht="75" customHeight="1">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>9.3</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>WP7 — Cross-platform Packaging</t>
+          <t>WP6 — Doc Processing Benchmarks</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Native Windows Service path</t>
+          <t>Build /benchmarks/ harness</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Purpose: support Windows Server native installs.
-Steps: Windows Service wrapper; SurrealDB-on-Windows notes; frontend serve docs; verify on Windows Server or equivalent.</t>
+          <t>Purpose: produce repeatable measured metrics — not estimates — for ingestion, extraction, embedding, memory, and search/chat latency.
+Steps: build parameterized harness under /benchmarks/; output machine-readable reports.</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>Windows native docs + scripts</t>
+          <t>/benchmarks/ harness</t>
         </is>
       </c>
       <c r="F86" s="22" t="inlineStr">
@@ -7679,21 +7802,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G86" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G86" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="I86" s="17" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="J86" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K86" s="17" t="n"/>
       <c r="L86" s="18" t="n">
@@ -7701,19 +7824,19 @@
       </c>
       <c r="M86" s="3" t="inlineStr">
         <is>
-          <t>DevOps / Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N86" s="19" t="n">
-        <v>46287</v>
+        <v>46267</v>
       </c>
       <c r="O86" s="19" t="n">
-        <v>46289</v>
+        <v>46270</v>
       </c>
       <c r="P86" s="3" t="n"/>
       <c r="Q86" s="3" t="inlineStr">
         <is>
-          <t>Verified on Windows Server or equivalent</t>
+          <t>Harness runs repeatably and outputs a metrics report</t>
         </is>
       </c>
       <c r="R86" s="3" t="inlineStr"/>
@@ -7722,28 +7845,28 @@
     <row r="87" ht="75" customHeight="1">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>WP7 — Cross-platform Packaging</t>
+          <t>WP6 — Doc Processing Benchmarks</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Installer helper CLI (interactive + non-interactive)</t>
+          <t>Assemble representative corpus</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Purpose: let a non-expert stand up a branded client instance without hand-editing half a dozen files.
-Steps: CLI for prereq check → collect brand/Entra/provider/DB/encryption → write config → migrate → start → health check; add scripted/non-interactive mode for repeatable installs.</t>
+          <t>Purpose: find empirical slowdown/failure points across sizes and types.
+Steps: assemble small/medium/large/very-large docs plus scanned PDF, audio, and web page; ensure corpus licensing is clean for redistribution in-repo if needed.</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>onboard/install CLI</t>
+          <t>Fixed corpus under benchmarks/</t>
         </is>
       </c>
       <c r="F87" s="22" t="inlineStr">
@@ -7751,21 +7874,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G87" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G87" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>9.1,5.4</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="I87" s="17" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="J87" s="17" t="n">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="K87" s="17" t="n"/>
       <c r="L87" s="18" t="n">
@@ -7773,53 +7896,49 @@
       </c>
       <c r="M87" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N87" s="19" t="n">
-        <v>46289</v>
+        <v>46270</v>
       </c>
       <c r="O87" s="19" t="n">
-        <v>46295</v>
+        <v>46273</v>
       </c>
       <c r="P87" s="3" t="n"/>
       <c r="Q87" s="3" t="inlineStr">
         <is>
-          <t>Full install in both modes; scripted branded client stand-up works</t>
-        </is>
-      </c>
-      <c r="R87" s="3" t="inlineStr">
-        <is>
-          <t>Deployment counterpart to WP3 theming</t>
-        </is>
-      </c>
+          <t>Corpus covers the size/type matrix</t>
+        </is>
+      </c>
+      <c r="R87" s="3" t="inlineStr"/>
       <c r="S87" s="3" t="inlineStr"/>
     </row>
     <row r="88" ht="75" customHeight="1">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>WP7 — Cross-platform Packaging</t>
+          <t>WP6 — Doc Processing Benchmarks</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>docs/DEPLOYMENT.md + WP7 review</t>
+          <t>Define accuracy methodology</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Purpose: one operator guide for container + native + CLI paths.
-Steps: write DEPLOYMENT.md; verify WP7 ACs; PR; human review.</t>
+          <t>Purpose: define how accuracy is measured so client claims are defensible.
+Steps: specify extraction fidelity, retrieval relevance (labeled Q&amp;A), and chat groundedness methods; report per model tier.</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>docs/DEPLOYMENT.md</t>
+          <t>Accuracy method doc section</t>
         </is>
       </c>
       <c r="F88" s="22" t="inlineStr">
@@ -7834,7 +7953,7 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>9.2,9.3,9.4</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="I88" s="17" t="n">
@@ -7853,15 +7972,15 @@
         </is>
       </c>
       <c r="N88" s="19" t="n">
-        <v>46295</v>
+        <v>46270</v>
       </c>
       <c r="O88" s="19" t="n">
-        <v>46296</v>
+        <v>46273</v>
       </c>
       <c r="P88" s="3" t="n"/>
       <c r="Q88" s="3" t="inlineStr">
         <is>
-          <t>All WP7 acceptance criteria pass</t>
+          <t>Accuracy reported as method + numbers</t>
         </is>
       </c>
       <c r="R88" s="3" t="inlineStr"/>
@@ -7870,28 +7989,28 @@
     <row r="89" ht="75" customHeight="1">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>WP8 — Onboarding &amp; In-app Help</t>
+          <t>WP6 — Doc Processing Benchmarks</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>WP8 kickoff (LAST)</t>
+          <t>Run ≥2 hardware profiles</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Purpose: build onboarding against final flows only — wizard/tour copy must match the shipped product.
-Steps: create wp-8-onboarding after WP2/3/5/7 are stable on main.</t>
+          <t>Purpose: gather real numbers on bare-minimum and recommended hardware.
+Steps: run harness on both profiles; record figures; note local-model vs API-provider resource differences. Requires access to target hardware.</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>Raw results JSON/CSV</t>
         </is>
       </c>
       <c r="F89" s="22" t="inlineStr">
@@ -7899,21 +8018,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G89" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G89" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>9.5,7.6,5.6</t>
+          <t>8.2,8.3</t>
         </is>
       </c>
       <c r="I89" s="17" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="J89" s="17" t="n">
-        <v>0.25</v>
+        <v>3</v>
       </c>
       <c r="K89" s="17" t="n"/>
       <c r="L89" s="18" t="n">
@@ -7921,24 +8040,24 @@
       </c>
       <c r="M89" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N89" s="19" t="n">
-        <v>46297</v>
+        <v>46273</v>
       </c>
       <c r="O89" s="19" t="n">
-        <v>46297</v>
+        <v>46276</v>
       </c>
       <c r="P89" s="3" t="n"/>
       <c r="Q89" s="3" t="inlineStr">
         <is>
-          <t>Built against final UX</t>
+          <t>Real measured numbers for both profiles</t>
         </is>
       </c>
       <c r="R89" s="3" t="inlineStr">
         <is>
-          <t>Must be last in the program sequence</t>
+          <t>Hardware access is a dependency</t>
         </is>
       </c>
       <c r="S89" s="3" t="inlineStr"/>
@@ -7946,28 +8065,28 @@
     <row r="90" ht="75" customHeight="1">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>WP8 — Onboarding &amp; In-app Help</t>
+          <t>WP6 — Doc Processing Benchmarks</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>First-run / admin setup wizard</t>
+          <t>docs/PERFORMANCE_AND_SIZING.md + review</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Purpose: take a fresh instance to a working configured app without tribal knowledge.
-Steps: detect fresh instance; guide providers/keys, models, brand (admin), connect a source, create first notebook; all copy via i18n.</t>
+          <t>Purpose: publish client-facing sizing guidance backed only by harness output.
+Steps: write types, limits, times, accuracy, min vs recommended hardware; peer review; merge.</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>Setup wizard</t>
+          <t>docs/PERFORMANCE_AND_SIZING.md</t>
         </is>
       </c>
       <c r="F90" s="22" t="inlineStr">
@@ -7982,14 +8101,14 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="I90" s="17" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="J90" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K90" s="17" t="n"/>
       <c r="L90" s="18" t="n">
@@ -7997,19 +8116,19 @@
       </c>
       <c r="M90" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N90" s="19" t="n">
-        <v>46297</v>
+        <v>46276</v>
       </c>
       <c r="O90" s="19" t="n">
-        <v>46302</v>
+        <v>46277</v>
       </c>
       <c r="P90" s="3" t="n"/>
       <c r="Q90" s="3" t="inlineStr">
         <is>
-          <t>Completing the wizard leaves a working configured app</t>
+          <t>Doc contains measured numbers only</t>
         </is>
       </c>
       <c r="R90" s="3" t="inlineStr"/>
@@ -8018,28 +8137,28 @@
     <row r="91" ht="75" customHeight="1">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>WP8 — Onboarding &amp; In-app Help</t>
+          <t>WP7 — Cross-platform Packaging</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>User guided tour (core loop)</t>
+          <t>WP7 kickoff</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Purpose: teach the core loop — add source → search → chat → transform → podcast — with an accessible spotlight tour.
-Steps: implement dismissible/resumable tour; keep steps short; i18n all locales.</t>
+          <t>Purpose: package the real authenticated + branded app, not the pre-WP2 password prototype.
+Steps: create wp-7-packaging only after WP2 and WP3 are on main.</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>Guided tour</t>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F91" s="22" t="inlineStr">
@@ -8054,14 +8173,14 @@
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>5.6,4.10</t>
         </is>
       </c>
       <c r="I91" s="17" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="J91" s="17" t="n">
-        <v>2</v>
+        <v>0.25</v>
       </c>
       <c r="K91" s="17" t="n"/>
       <c r="L91" s="18" t="n">
@@ -8069,19 +8188,19 @@
       </c>
       <c r="M91" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N91" s="19" t="n">
-        <v>46302</v>
+        <v>46283</v>
       </c>
       <c r="O91" s="19" t="n">
-        <v>46304</v>
+        <v>46283</v>
       </c>
       <c r="P91" s="3" t="n"/>
       <c r="Q91" s="3" t="inlineStr">
         <is>
-          <t>New user can complete the core-loop tour</t>
+          <t>Starts only after branded + authenticated app exists</t>
         </is>
       </c>
       <c r="R91" s="3" t="inlineStr"/>
@@ -8090,28 +8209,28 @@
     <row r="92" ht="75" customHeight="1">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>WP8 — Onboarding &amp; In-app Help</t>
+          <t>WP7 — Cross-platform Packaging</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Contextual tooltips + empty states + help surface</t>
+          <t>Verify Docker Compose on Windows + Linux</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Purpose: remove dead-ends for new users on every main screen.
-Steps: tooltips on non-obvious controls; useful empty states; persistent help (docs, shortcuts, restart tour, BrandConfig support URL); all strings in i18n.</t>
+          <t>Purpose: make containers the recommended identical path on both OSes.
+Steps: verify docker-compose and Dockerfile.single on Docker Desktop/WSL2 and Linux; document as primary deploy path.</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>Tooltips/empty states/help</t>
+          <t>Verified container deploy</t>
         </is>
       </c>
       <c r="F92" s="22" t="inlineStr">
@@ -8119,21 +8238,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G92" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G92" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="I92" s="17" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J92" s="17" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="K92" s="17" t="n"/>
       <c r="L92" s="18" t="n">
@@ -8141,53 +8260,49 @@
       </c>
       <c r="M92" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>DevOps / Engineer</t>
         </is>
       </c>
       <c r="N92" s="19" t="n">
-        <v>46304</v>
+        <v>46283</v>
       </c>
       <c r="O92" s="19" t="n">
-        <v>46309</v>
+        <v>46287</v>
       </c>
       <c r="P92" s="3" t="n"/>
       <c r="Q92" s="3" t="inlineStr">
         <is>
-          <t>All copy in i18n; help reachable everywhere</t>
-        </is>
-      </c>
-      <c r="R92" s="3" t="inlineStr">
-        <is>
-          <t>Locale parity required across all locales</t>
-        </is>
-      </c>
+          <t>Container deployment verified on both OSes</t>
+        </is>
+      </c>
+      <c r="R92" s="3" t="inlineStr"/>
       <c r="S92" s="3" t="inlineStr"/>
     </row>
     <row r="93" ht="75" customHeight="1">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>WP8 — Onboarding &amp; In-app Help</t>
+          <t>WP7 — Cross-platform Packaging</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>docs/ONBOARDING.md + program close review</t>
+          <t>Native Linux install path (systemd)</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Purpose: document onboarding structure and verify program-level definition of done.
-Steps: write ONBOARDING.md; confirm a new client can be stood up by config + installer only (branded, Entra-auth’d, connectors, Windows/Linux) without per-client code rebuilds.</t>
+          <t>Purpose: support customers who refuse containers.
+Steps: systemd units + install script; document dependencies for common distros; verify on at least one distro.</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>docs/ONBOARDING.md; program DoD check</t>
+          <t>Linux native docs + scripts</t>
         </is>
       </c>
       <c r="F93" s="22" t="inlineStr">
@@ -8202,14 +8317,14 @@
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="I93" s="17" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="J93" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K93" s="17" t="n"/>
       <c r="L93" s="18" t="n">
@@ -8217,26 +8332,614 @@
       </c>
       <c r="M93" s="3" t="inlineStr">
         <is>
-          <t>Engineering Lead</t>
+          <t>DevOps / Engineer</t>
         </is>
       </c>
       <c r="N93" s="19" t="n">
-        <v>46309</v>
+        <v>46287</v>
       </c>
       <c r="O93" s="19" t="n">
-        <v>46310</v>
+        <v>46289</v>
       </c>
       <c r="P93" s="3" t="n"/>
       <c r="Q93" s="3" t="inlineStr">
         <is>
-          <t>All WP8 ACs + program definition of done satisfied</t>
+          <t>Verified on ≥1 Linux distro</t>
         </is>
       </c>
       <c r="R93" s="3" t="inlineStr"/>
       <c r="S93" s="3" t="inlineStr"/>
     </row>
+    <row r="94" ht="75" customHeight="1">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>WP7 — Cross-platform Packaging</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Native Windows Service path</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: support Windows Server native installs.
+Steps: Windows Service wrapper; SurrealDB-on-Windows notes; frontend serve docs; verify on Windows Server or equivalent.</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>Windows native docs + scripts</t>
+        </is>
+      </c>
+      <c r="F94" s="22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G94" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="I94" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="J94" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K94" s="17" t="n"/>
+      <c r="L94" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M94" s="3" t="inlineStr">
+        <is>
+          <t>DevOps / Engineer</t>
+        </is>
+      </c>
+      <c r="N94" s="19" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O94" s="19" t="n">
+        <v>46289</v>
+      </c>
+      <c r="P94" s="3" t="n"/>
+      <c r="Q94" s="3" t="inlineStr">
+        <is>
+          <t>Verified on Windows Server or equivalent</t>
+        </is>
+      </c>
+      <c r="R94" s="3" t="inlineStr"/>
+      <c r="S94" s="3" t="inlineStr"/>
+    </row>
+    <row r="95" ht="75" customHeight="1">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>WP7 — Cross-platform Packaging</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Installer helper CLI (interactive + non-interactive)</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: let a non-expert stand up a branded client instance without hand-editing half a dozen files.
+Steps: CLI for prereq check → collect brand/Entra/provider/DB/encryption → write config → migrate → start → health check; add scripted/non-interactive mode for repeatable installs.</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>onboard/install CLI</t>
+        </is>
+      </c>
+      <c r="F95" s="22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G95" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="H95" s="3" t="inlineStr">
+        <is>
+          <t>9.1,5.4</t>
+        </is>
+      </c>
+      <c r="I95" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="J95" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K95" s="17" t="n"/>
+      <c r="L95" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M95" s="3" t="inlineStr">
+        <is>
+          <t>Backend Engineer</t>
+        </is>
+      </c>
+      <c r="N95" s="19" t="n">
+        <v>46289</v>
+      </c>
+      <c r="O95" s="19" t="n">
+        <v>46295</v>
+      </c>
+      <c r="P95" s="3" t="n"/>
+      <c r="Q95" s="3" t="inlineStr">
+        <is>
+          <t>Full install in both modes; scripted branded client stand-up works</t>
+        </is>
+      </c>
+      <c r="R95" s="3" t="inlineStr">
+        <is>
+          <t>Deployment counterpart to WP3 theming</t>
+        </is>
+      </c>
+      <c r="S95" s="3" t="inlineStr"/>
+    </row>
+    <row r="96" ht="75" customHeight="1">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>WP7 — Cross-platform Packaging</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>docs/DEPLOYMENT.md + WP7 review</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: one operator guide for container + native + CLI paths.
+Steps: write DEPLOYMENT.md; verify WP7 ACs; PR; human review.</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>docs/DEPLOYMENT.md</t>
+        </is>
+      </c>
+      <c r="F96" s="22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G96" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>9.2,9.3,9.4</t>
+        </is>
+      </c>
+      <c r="I96" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="J96" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K96" s="17" t="n"/>
+      <c r="L96" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M96" s="3" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="N96" s="19" t="n">
+        <v>46295</v>
+      </c>
+      <c r="O96" s="19" t="n">
+        <v>46296</v>
+      </c>
+      <c r="P96" s="3" t="n"/>
+      <c r="Q96" s="3" t="inlineStr">
+        <is>
+          <t>All WP7 acceptance criteria pass</t>
+        </is>
+      </c>
+      <c r="R96" s="3" t="inlineStr"/>
+      <c r="S96" s="3" t="inlineStr"/>
+    </row>
+    <row r="97" ht="75" customHeight="1">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>WP8 — Onboarding &amp; In-app Help</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>WP8 kickoff (LAST)</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: build onboarding against final flows only — wizard/tour copy must match the shipped product.
+Steps: create wp-8-onboarding after WP2/3/5/7 are stable on main.</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="F97" s="22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G97" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H97" s="3" t="inlineStr">
+        <is>
+          <t>9.5,7.6,5.6</t>
+        </is>
+      </c>
+      <c r="I97" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="J97" s="17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K97" s="17" t="n"/>
+      <c r="L97" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M97" s="3" t="inlineStr">
+        <is>
+          <t>Frontend Engineer</t>
+        </is>
+      </c>
+      <c r="N97" s="19" t="n">
+        <v>46297</v>
+      </c>
+      <c r="O97" s="19" t="n">
+        <v>46297</v>
+      </c>
+      <c r="P97" s="3" t="n"/>
+      <c r="Q97" s="3" t="inlineStr">
+        <is>
+          <t>Built against final UX</t>
+        </is>
+      </c>
+      <c r="R97" s="3" t="inlineStr">
+        <is>
+          <t>Must be last in the program sequence</t>
+        </is>
+      </c>
+      <c r="S97" s="3" t="inlineStr"/>
+    </row>
+    <row r="98" ht="75" customHeight="1">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>WP8 — Onboarding &amp; In-app Help</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>First-run / admin setup wizard</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: take a fresh instance to a working configured app without tribal knowledge.
+Steps: detect fresh instance; guide providers/keys, models, brand (admin), connect a source, create first notebook; all copy via i18n.</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>Setup wizard</t>
+        </is>
+      </c>
+      <c r="F98" s="22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G98" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H98" s="3" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="I98" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="J98" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K98" s="17" t="n"/>
+      <c r="L98" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M98" s="3" t="inlineStr">
+        <is>
+          <t>Frontend Engineer</t>
+        </is>
+      </c>
+      <c r="N98" s="19" t="n">
+        <v>46297</v>
+      </c>
+      <c r="O98" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="P98" s="3" t="n"/>
+      <c r="Q98" s="3" t="inlineStr">
+        <is>
+          <t>Completing the wizard leaves a working configured app</t>
+        </is>
+      </c>
+      <c r="R98" s="3" t="inlineStr"/>
+      <c r="S98" s="3" t="inlineStr"/>
+    </row>
+    <row r="99" ht="75" customHeight="1">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>WP8 — Onboarding &amp; In-app Help</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>User guided tour (core loop)</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: teach the core loop — add source → search → chat → transform → podcast — with an accessible spotlight tour.
+Steps: implement dismissible/resumable tour; keep steps short; i18n all locales.</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>Guided tour</t>
+        </is>
+      </c>
+      <c r="F99" s="22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G99" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H99" s="3" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="I99" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="J99" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K99" s="17" t="n"/>
+      <c r="L99" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M99" s="3" t="inlineStr">
+        <is>
+          <t>Frontend Engineer</t>
+        </is>
+      </c>
+      <c r="N99" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="O99" s="19" t="n">
+        <v>46304</v>
+      </c>
+      <c r="P99" s="3" t="n"/>
+      <c r="Q99" s="3" t="inlineStr">
+        <is>
+          <t>New user can complete the core-loop tour</t>
+        </is>
+      </c>
+      <c r="R99" s="3" t="inlineStr"/>
+      <c r="S99" s="3" t="inlineStr"/>
+    </row>
+    <row r="100" ht="75" customHeight="1">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>WP8 — Onboarding &amp; In-app Help</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>Contextual tooltips + empty states + help surface</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: remove dead-ends for new users on every main screen.
+Steps: tooltips on non-obvious controls; useful empty states; persistent help (docs, shortcuts, restart tour, BrandConfig support URL); all strings in i18n.</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>Tooltips/empty states/help</t>
+        </is>
+      </c>
+      <c r="F100" s="22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G100" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H100" s="3" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="I100" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="J100" s="17" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K100" s="17" t="n"/>
+      <c r="L100" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M100" s="3" t="inlineStr">
+        <is>
+          <t>Frontend Engineer</t>
+        </is>
+      </c>
+      <c r="N100" s="19" t="n">
+        <v>46304</v>
+      </c>
+      <c r="O100" s="19" t="n">
+        <v>46309</v>
+      </c>
+      <c r="P100" s="3" t="n"/>
+      <c r="Q100" s="3" t="inlineStr">
+        <is>
+          <t>All copy in i18n; help reachable everywhere</t>
+        </is>
+      </c>
+      <c r="R100" s="3" t="inlineStr">
+        <is>
+          <t>Locale parity required across all locales</t>
+        </is>
+      </c>
+      <c r="S100" s="3" t="inlineStr"/>
+    </row>
+    <row r="101" ht="75" customHeight="1">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>10.4</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>WP8 — Onboarding &amp; In-app Help</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>docs/ONBOARDING.md + program close review</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: document onboarding structure and verify program-level definition of done.
+Steps: write ONBOARDING.md; confirm a new client can be stood up by config + installer only (branded, Entra-auth’d, connectors, Windows/Linux) without per-client code rebuilds.</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>docs/ONBOARDING.md; program DoD check</t>
+        </is>
+      </c>
+      <c r="F101" s="22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G101" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H101" s="3" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="I101" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="J101" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K101" s="17" t="n"/>
+      <c r="L101" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M101" s="3" t="inlineStr">
+        <is>
+          <t>Engineering Lead</t>
+        </is>
+      </c>
+      <c r="N101" s="19" t="n">
+        <v>46309</v>
+      </c>
+      <c r="O101" s="19" t="n">
+        <v>46310</v>
+      </c>
+      <c r="P101" s="3" t="n"/>
+      <c r="Q101" s="3" t="inlineStr">
+        <is>
+          <t>All WP8 ACs + program definition of done satisfied</t>
+        </is>
+      </c>
+      <c r="R101" s="3" t="inlineStr"/>
+      <c r="S101" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:S93"/>
+  <autoFilter ref="A5:S101"/>
   <mergeCells count="3">
     <mergeCell ref="A3:S3"/>
     <mergeCell ref="A2:S2"/>
@@ -8307,7 +9010,7 @@
           <t>Clean build reproducible from docs/DEV_SETUP.md</t>
         </is>
       </c>
-      <c r="C4" s="25" t="inlineStr">
+      <c r="C4" s="26" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8330,7 +9033,7 @@
           <t>upstream-base tag exists; upstream remote configured</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8357,7 +9060,7 @@
           <t>Characterization tests: ingestion, search, chat, notebook CRUD</t>
         </is>
       </c>
-      <c r="C6" s="25" t="inlineStr">
+      <c r="C6" s="26" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8380,7 +9083,7 @@
           <t>CI runs on PR and blocks merge on failure</t>
         </is>
       </c>
-      <c r="C7" s="25" t="inlineStr">
+      <c r="C7" s="26" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8403,7 +9106,7 @@
           <t>License scan runs in CI and passes</t>
         </is>
       </c>
-      <c r="C8" s="25" t="inlineStr">
+      <c r="C8" s="26" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8426,7 +9129,7 @@
           <t>LICENSE retains upstream copyright + our copyright</t>
         </is>
       </c>
-      <c r="C9" s="25" t="inlineStr">
+      <c r="C9" s="26" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8453,7 +9156,7 @@
           <t>THIRD-PARTY-NOTICES.md complete and reproducible</t>
         </is>
       </c>
-      <c r="C10" s="25" t="inlineStr">
+      <c r="C10" s="26" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8480,7 +9183,7 @@
           <t>SurrealDB BSL entry present and accurate</t>
         </is>
       </c>
-      <c r="C11" s="25" t="inlineStr">
+      <c r="C11" s="26" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8503,7 +9206,7 @@
           <t>pycountry unmodified; CI asserts</t>
         </is>
       </c>
-      <c r="C12" s="25" t="inlineStr">
+      <c r="C12" s="26" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8526,7 +9229,7 @@
           <t>docs/PROVIDER_TERMS.md exists</t>
         </is>
       </c>
-      <c r="C13" s="25" t="inlineStr">
+      <c r="C13" s="26" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8553,7 +9256,7 @@
           <t>No secrets committed; encryption key handling documented</t>
         </is>
       </c>
-      <c r="C14" s="25" t="inlineStr">
+      <c r="C14" s="26" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8576,7 +9279,7 @@
           <t>Tenancy model chosen and documented</t>
         </is>
       </c>
-      <c r="C15" s="25" t="inlineStr">
+      <c r="C15" s="26" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8603,7 +9306,7 @@
           <t>Login via real Entra account E2E</t>
         </is>
       </c>
-      <c r="C16" s="26" t="inlineStr">
+      <c r="C16" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8626,7 +9329,7 @@
           <t>Every API request validates Entra JWT (iss/aud/sig/exp)</t>
         </is>
       </c>
-      <c r="C17" s="26" t="inlineStr">
+      <c r="C17" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8645,7 +9348,7 @@
           <t>Users JIT-provisioned; user record after first login</t>
         </is>
       </c>
-      <c r="C18" s="26" t="inlineStr">
+      <c r="C18" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8664,7 +9367,7 @@
           <t>Roles enforced on sensitive routes (403)</t>
         </is>
       </c>
-      <c r="C19" s="26" t="inlineStr">
+      <c r="C19" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8683,7 +9386,7 @@
           <t>Users only see own notebooks/sources</t>
         </is>
       </c>
-      <c r="C20" s="26" t="inlineStr">
+      <c r="C20" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8702,7 +9405,7 @@
           <t>Password provider still works as local-dev fallback</t>
         </is>
       </c>
-      <c r="C21" s="26" t="inlineStr">
+      <c r="C21" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8721,7 +9424,7 @@
           <t>Second provider needs no route-handler changes (stub)</t>
         </is>
       </c>
-      <c r="C22" s="26" t="inlineStr">
+      <c r="C22" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8740,7 +9443,7 @@
           <t>docs/AUTH.md complete</t>
         </is>
       </c>
-      <c r="C23" s="26" t="inlineStr">
+      <c r="C23" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8759,7 +9462,7 @@
           <t>FRONTEND_MAP.md complete with where-to-change table</t>
         </is>
       </c>
-      <c r="C24" s="26" t="inlineStr">
+      <c r="C24" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8778,7 +9481,7 @@
           <t>New client branded by config only (two brands, same build)</t>
         </is>
       </c>
-      <c r="C25" s="26" t="inlineStr">
+      <c r="C25" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8797,7 +9500,7 @@
           <t>Hardcoded brand strings/assets read from BrandConfig</t>
         </is>
       </c>
-      <c r="C26" s="26" t="inlineStr">
+      <c r="C26" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8816,7 +9519,7 @@
           <t>Dark/light both themed correctly</t>
         </is>
       </c>
-      <c r="C27" s="26" t="inlineStr">
+      <c r="C27" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8835,7 +9538,7 @@
           <t>Every router/endpoint documented with auth + models</t>
         </is>
       </c>
-      <c r="C28" s="26" t="inlineStr">
+      <c r="C28" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8854,7 +9557,7 @@
           <t>Every domain model and graph documented</t>
         </is>
       </c>
-      <c r="C29" s="26" t="inlineStr">
+      <c r="C29" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8873,7 +9576,7 @@
           <t>Five how-to-add-X playbooks present</t>
         </is>
       </c>
-      <c r="C30" s="26" t="inlineStr">
+      <c r="C30" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8892,7 +9595,7 @@
           <t>New engineer can locate changes using only BACKEND_MAP</t>
         </is>
       </c>
-      <c r="C31" s="26" t="inlineStr">
+      <c r="C31" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8911,7 +9614,7 @@
           <t>SharePoint connect → folder → pull all supported docs</t>
         </is>
       </c>
-      <c r="C32" s="26" t="inlineStr">
+      <c r="C32" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8930,7 +9633,7 @@
           <t>Ingestion reuses existing pipeline</t>
         </is>
       </c>
-      <c r="C33" s="26" t="inlineStr">
+      <c r="C33" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8949,7 +9652,7 @@
           <t>Batch per-doc progress; single failure non-fatal</t>
         </is>
       </c>
-      <c r="C34" s="26" t="inlineStr">
+      <c r="C34" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8968,7 +9671,7 @@
           <t>Chat across whole pulled set</t>
         </is>
       </c>
-      <c r="C35" s="26" t="inlineStr">
+      <c r="C35" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -8987,7 +9690,7 @@
           <t>Tokens encrypted per user; source permissions respected</t>
         </is>
       </c>
-      <c r="C36" s="26" t="inlineStr">
+      <c r="C36" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9006,7 +9709,7 @@
           <t>New connector = SourceConnector interface only</t>
         </is>
       </c>
-      <c r="C37" s="26" t="inlineStr">
+      <c r="C37" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9025,7 +9728,7 @@
           <t>docs/CONNECTORS.md complete</t>
         </is>
       </c>
-      <c r="C38" s="26" t="inlineStr">
+      <c r="C38" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9044,7 +9747,7 @@
           <t>Benchmark harness repeatable with metrics report</t>
         </is>
       </c>
-      <c r="C39" s="26" t="inlineStr">
+      <c r="C39" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9063,7 +9766,7 @@
           <t>PERFORMANCE_AND_SIZING.md has measured numbers (2 profiles)</t>
         </is>
       </c>
-      <c r="C40" s="26" t="inlineStr">
+      <c r="C40" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9082,7 +9785,7 @@
           <t>Supported types + tested size limits + failure points</t>
         </is>
       </c>
-      <c r="C41" s="26" t="inlineStr">
+      <c r="C41" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9101,7 +9804,7 @@
           <t>Accuracy methodology + results per model tier</t>
         </is>
       </c>
-      <c r="C42" s="26" t="inlineStr">
+      <c r="C42" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9120,7 +9823,7 @@
           <t>Min vs recommended hardware justified by numbers</t>
         </is>
       </c>
-      <c r="C43" s="26" t="inlineStr">
+      <c r="C43" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9139,7 +9842,7 @@
           <t>Container deploy verified Windows + Linux</t>
         </is>
       </c>
-      <c r="C44" s="26" t="inlineStr">
+      <c r="C44" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9158,7 +9861,7 @@
           <t>Native install documented/verified Linux + Windows</t>
         </is>
       </c>
-      <c r="C45" s="26" t="inlineStr">
+      <c r="C45" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9177,7 +9880,7 @@
           <t>Installer CLI full install interactive + non-interactive</t>
         </is>
       </c>
-      <c r="C46" s="26" t="inlineStr">
+      <c r="C46" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9196,7 +9899,7 @@
           <t>Scripted install stands up branded client E2E</t>
         </is>
       </c>
-      <c r="C47" s="26" t="inlineStr">
+      <c r="C47" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9215,7 +9918,7 @@
           <t>docs/DEPLOYMENT.md complete</t>
         </is>
       </c>
-      <c r="C48" s="26" t="inlineStr">
+      <c r="C48" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9234,7 +9937,7 @@
           <t>Fresh instance launches setup wizard → working app</t>
         </is>
       </c>
-      <c r="C49" s="26" t="inlineStr">
+      <c r="C49" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9253,7 +9956,7 @@
           <t>Guided tour of core loop completable</t>
         </is>
       </c>
-      <c r="C50" s="26" t="inlineStr">
+      <c r="C50" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9272,7 +9975,7 @@
           <t>Contextual tooltips; all copy in i18n</t>
         </is>
       </c>
-      <c r="C51" s="26" t="inlineStr">
+      <c r="C51" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9291,7 +9994,7 @@
           <t>Every main screen useful empty state</t>
         </is>
       </c>
-      <c r="C52" s="26" t="inlineStr">
+      <c r="C52" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9310,7 +10013,7 @@
           <t>Tour dismissible/resumable; help surface everywhere</t>
         </is>
       </c>
-      <c r="C53" s="26" t="inlineStr">
+      <c r="C53" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9329,7 +10032,7 @@
           <t>docs/ONBOARDING.md complete</t>
         </is>
       </c>
-      <c r="C54" s="26" t="inlineStr">
+      <c r="C54" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9348,7 +10051,7 @@
           <t>New client by config + installer only (no per-client rebuild)</t>
         </is>
       </c>
-      <c r="C55" s="26" t="inlineStr">
+      <c r="C55" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9371,7 +10074,7 @@
           <t>Licensing compliant and drift-guarded</t>
         </is>
       </c>
-      <c r="C56" s="25" t="inlineStr">
+      <c r="C56" s="26" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9394,7 +10097,7 @@
           <t>Real performance/sizing numbers for clients</t>
         </is>
       </c>
-      <c r="C57" s="26" t="inlineStr">
+      <c r="C57" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9417,7 +10120,7 @@
           <t>Backend + frontend fully mapped</t>
         </is>
       </c>
-      <c r="C58" s="26" t="inlineStr">
+      <c r="C58" s="27" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9458,12 +10161,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="27" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>Topic</t>
         </is>
       </c>
-      <c r="B3" s="27" t="inlineStr">
+      <c r="B3" s="28" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>

</xml_diff>